<commit_message>
docs(test): update results and remove personal data
</commit_message>
<xml_diff>
--- a/docs/testing-strategy/kiwishare-release-test-results-v0.2.xlsx
+++ b/docs/testing-strategy/kiwishare-release-test-results-v0.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra10e6dbd2e3d4a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data &amp; Setup" sheetId="2" r:id="Rfaa681c271dc4c06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="Rfa5341b623cd40d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="Rd6ff77a5a8d349ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdd307d4777844405"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data &amp; Setup" sheetId="2" r:id="R201d8dcc24af4d16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="R882edabbf8e04efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R2dc9307139ac4bc0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,6 +13,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
+    <x:t xml:space="preserve">KiwiShare — Release Test Plan / UAT Checklist (v0.2)</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">1. Test Object</x:t>
   </x:si>
   <x:si>
@@ -215,6 +218,36 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">100% P0 Pass; P1 Pass or accepted deferral; zero open S1/S2 defects; all evidence linked.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">9. Automated Regression Evidence</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Local pre-push run on 2026-10-02</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Flutter tests</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">451 passed; 0 failed</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Server Jest</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">24 test suites passed; 264 tests passed; 0 failed</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Source revision</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">docs/consolidated-test-evidence based on origin/pre 8bcb615</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Web evidence gap</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Web tests are not included in test:all; retain manual and CI evidence separately.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Test Data &amp; Environment Setup — do this BEFORE Round 1</x:t>
@@ -403,6 +436,45 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Replace with friendly message</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">KS-B-002</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">KS-T-013</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Profile</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Registration accepted display names longer than 30 characters while Profile editing capped them at 30.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Register with a 32-character nickname, then edit the nickname in Profile and enter a 33rd character.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Closed</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Fixed in PR #309 by applying the 2-30 character limit consistently; the linked test case now passes.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">KS-B-003</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">KS-T-008</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Floating labels overlapped adjacent fields in the change-password dialog.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Open Profile &gt; Change password and inspect spacing between the three password fields.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">S4 Cosmetic</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Fixed in PR #309 by restoring spacing between fields; the linked test case now passes.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -410,10 +482,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="2">
-    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
-    <x:numFmt numFmtId="201" formatCode="0.0%"/>
+    <x:numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <x:numFmt numFmtId="165" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -443,6 +515,7 @@
     </x:font>
     <x:font>
       <x:b/>
+      <x:sz val="11"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
       <x:scheme val="minor"/>
@@ -454,11 +527,13 @@
     </x:font>
     <x:font>
       <x:b/>
+      <x:sz val="11"/>
       <x:color rgb="FFC00000"/>
       <x:name val="Calibri"/>
       <x:scheme val="minor"/>
     </x:font>
     <x:font>
+      <x:sz val="11"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
       <x:scheme val="minor"/>
@@ -476,13 +551,19 @@
       <x:name val="Calibri"/>
       <x:scheme val="minor"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
   <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
-      <x:patternFill patternType="lightGray"/>
+      <x:patternFill patternType="gray125"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -496,7 +577,13 @@
     </x:fill>
   </x:fills>
   <x:borders count="2">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFBBBBBB"/>
@@ -510,88 +597,68 @@
       <x:bottom style="thin">
         <x:color rgb="FFBBBBBB"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="0" shrinkToFit="0"/>
-    </x:xf>
+  <x:cellXfs count="25">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1" shrinkToFit="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="0"/>
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="0"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="0"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="0"/>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="bottom" wrapText="1"/>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -602,21 +669,38 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="9">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFEB9C"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFEB9C"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
-      <x:border/>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
@@ -624,7 +708,13 @@
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
-      <x:border/>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF2F2F2"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
@@ -632,15 +722,20 @@
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
-      <x:border/>
     </x:dxf>
     <x:dxf>
       <x:fill>
         <x:patternFill>
-          <x:bgColor rgb="FFF2F2F2"/>
+          <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
-      <x:border/>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
@@ -839,424 +934,424 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultColWidth="14.430000305175781" defaultRowHeight="15"/>
+  <x:sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="78" hidden="0" customWidth="1"/>
-    <x:col min="3" max="26" width="8.710000038146973" customWidth="1"/>
+    <x:col min="1" max="1" width="30" customWidth="1"/>
+    <x:col min="2" max="2" width="78" customWidth="1"/>
+    <x:col min="3" max="26" width="8.6640625" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
-        <x:v>KiwiShare — Release Test Plan / UAT Checklist (v0.2)</x:v>
+    <x:row r="1" ht="19">
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="16">
       <x:c r="A4" s="4" t="s">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="16">
       <x:c r="A5" s="4" t="s">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="32">
       <x:c r="A6" s="4" t="s">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="16">
       <x:c r="A7" s="4" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="32">
       <x:c r="A8" s="4" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="32">
       <x:c r="A9" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="3" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="32">
       <x:c r="A12" s="4" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="16">
       <x:c r="A13" s="4" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="32">
       <x:c r="A14" s="4" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="16">
       <x:c r="A15" s="4" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="16">
       <x:c r="A18" s="4" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="16">
       <x:c r="A19" s="4" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="16">
       <x:c r="A20" s="4" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="4" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
       <x:c r="A22" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="4" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="4" t="s">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1"/>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="3" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="4" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="4" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B29" s="5" t="s">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="4" t="s">
-        <x:v>44</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B30" s="5" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15.75" customHeight="1">
       <x:c r="A31" s="4" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B31" s="5" t="s">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15.75" customHeight="1">
       <x:c r="A32" s="4" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B32" s="5" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1"/>
     <x:row r="34" ht="15.75" customHeight="1">
       <x:c r="A34" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
       <x:c r="A35" s="4" t="s">
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B35" s="5" t="s">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
       <x:c r="A36" s="4" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B36" s="5" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15.75" customHeight="1">
       <x:c r="A37" s="4" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B37" s="5" t="s">
-        <x:v>55</x:v>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15.75" customHeight="1"/>
     <x:row r="39" ht="15.75" customHeight="1">
       <x:c r="A39" s="3" t="s">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15.75" customHeight="1">
       <x:c r="A40" s="4" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B40" s="5" t="s">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15.75" customHeight="1">
       <x:c r="A41" s="4" t="s">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B41" s="5" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15.75" customHeight="1">
       <x:c r="A42" s="4" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B42" s="5" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15.75" customHeight="1"/>
     <x:row r="44" ht="15.75" customHeight="1">
       <x:c r="A44" s="3" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15.75" customHeight="1">
       <x:c r="A45" s="4" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B45" s="5" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15.75" customHeight="1">
       <x:c r="A46" s="4" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B46" s="5" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
-      <x:c r="A47" s="29" t="str">
+      <x:c r="A47" s="22" t="str">
         <x:v>8. Consolidated Test Results</x:v>
       </x:c>
-      <x:c r="B47" s="29" t="str">
-        <x:v>As of 2026-09-19</x:v>
+      <x:c r="B47" s="22" t="str">
+        <x:v>As of 2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
-      <x:c r="A48" s="30" t="str">
+      <x:c r="A48" s="23" t="str">
         <x:v>Total test cases</x:v>
       </x:c>
-      <x:c r="B48" s="31" t="n">
+      <x:c r="B48" s="24" t="n">
         <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
-      <x:c r="A49" s="30" t="str">
+      <x:c r="A49" s="23" t="str">
         <x:v>Executed</x:v>
       </x:c>
-      <x:c r="B49" s="31" t="n">
-        <x:v>33</x:v>
+      <x:c r="B49" s="24" t="n">
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
-      <x:c r="A50" s="30" t="str">
+      <x:c r="A50" s="23" t="str">
         <x:v>Passed</x:v>
       </x:c>
-      <x:c r="B50" s="31" t="n">
-        <x:v>28</x:v>
+      <x:c r="B50" s="24" t="n">
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
-      <x:c r="A51" s="30" t="str">
+      <x:c r="A51" s="23" t="str">
         <x:v>Failed</x:v>
       </x:c>
-      <x:c r="B51" s="31" t="n">
-        <x:v>5</x:v>
+      <x:c r="B51" s="24" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
-      <x:c r="A52" s="30" t="str">
+      <x:c r="A52" s="23" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="B52" s="31" t="n">
+      <x:c r="B52" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
-      <x:c r="A53" s="30" t="str">
+      <x:c r="A53" s="23" t="str">
         <x:v>Execution rate</x:v>
       </x:c>
-      <x:c r="B53" s="32" t="n">
-        <x:v>0.4714285714285714</x:v>
+      <x:c r="B53" s="21" t="n">
+        <x:v>0.7857142857142857</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
-      <x:c r="A54" s="30" t="str">
+      <x:c r="A54" s="23" t="str">
         <x:v>Pass rate (executed cases)</x:v>
       </x:c>
-      <x:c r="B54" s="32" t="n">
-        <x:v>0.8484848484848485</x:v>
+      <x:c r="B54" s="21" t="n">
+        <x:v>0.9272727272727272</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
-      <x:c r="A55" s="30" t="str">
-        <x:v>Imported source</x:v>
-      </x:c>
-      <x:c r="B55" s="31" t="str">
-        <x:v>26 results completed by Rui / Sam in the Chinese test plan on 2026-09-19.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="15" hidden="0" customHeight="1">
-      <x:c r="A56" s="30" t="str">
+      <x:c r="A55" s="23" t="str">
+        <x:v>Latest update</x:v>
+      </x:c>
+      <x:c r="B55" s="24" t="str">
+        <x:v>Results updated by the team on 2026-10-02; 15 cases remain Not run.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A56" s="23" t="str">
         <x:v>Evidence limitation</x:v>
       </x:c>
-      <x:c r="B56" s="31" t="str">
-        <x:v>Five failed cases still require linked GitHub defect IDs and retest evidence.</x:v>
+      <x:c r="B56" s="24" t="str">
+        <x:v>4 failed cases require linked GitHub defects; 29 executed cases still need complete tester/date metadata or evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15.75" customHeight="1"/>
-    <x:row r="58" ht="15" hidden="0" customHeight="1">
-      <x:c r="A58" s="29" t="str">
-        <x:v>9. Automated Regression Evidence</x:v>
-      </x:c>
-      <x:c r="B58" s="29" t="str">
-        <x:v>Local pre-push run on 2026-10-02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="15" hidden="0" customHeight="1">
-      <x:c r="A59" s="30" t="str">
-        <x:v>Flutter tests</x:v>
-      </x:c>
-      <x:c r="B59" s="31" t="str">
-        <x:v>451 passed; 0 failed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="15" hidden="0" customHeight="1">
-      <x:c r="A60" s="30" t="str">
-        <x:v>Server Jest</x:v>
-      </x:c>
-      <x:c r="B60" s="31" t="str">
-        <x:v>24 test suites passed; 264 tests passed; 0 failed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="15" hidden="0" customHeight="1">
-      <x:c r="A61" s="30" t="str">
-        <x:v>Source revision</x:v>
-      </x:c>
-      <x:c r="B61" s="31" t="str">
-        <x:v>docs/consolidated-test-evidence based on origin/pre 8bcb615</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="15" hidden="0" customHeight="1">
-      <x:c r="A62" s="30" t="str">
-        <x:v>Web evidence gap</x:v>
-      </x:c>
-      <x:c r="B62" s="31" t="str">
-        <x:v>Web tests are not included in test:all; retain manual and CI evidence separately.</x:v>
+    <x:row r="58" ht="15" customHeight="1">
+      <x:c r="A58" s="15" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B58" s="15" t="s">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="15" customHeight="1">
+      <x:c r="A59" s="16" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B59" s="17" t="s">
+        <x:v>72</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="15" customHeight="1">
+      <x:c r="A60" s="16" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B60" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="15" customHeight="1">
+      <x:c r="A61" s="16" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B61" s="17" t="s">
+        <x:v>76</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="15" customHeight="1">
+      <x:c r="A62" s="16" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B62" s="17" t="s">
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="15.75" customHeight="1"/>
@@ -2204,157 +2299,157 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultColWidth="14.430000305175781" defaultRowHeight="15"/>
+  <x:sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="26" customWidth="1"/>
     <x:col min="2" max="2" width="100" customWidth="1"/>
-    <x:col min="3" max="26" width="8.710000038146973" customWidth="1"/>
+    <x:col min="3" max="26" width="8.6640625" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="19">
       <x:c r="A1" s="1" t="s">
-        <x:v>68</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>69</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="16">
       <x:c r="A4" s="4" t="s">
-        <x:v>70</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>71</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+        <x:v>82</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="16">
       <x:c r="A5" s="4" t="s">
-        <x:v>72</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+        <x:v>84</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="16">
       <x:c r="A6" s="4" t="s">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>75</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+        <x:v>86</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="32">
       <x:c r="A7" s="4" t="s">
-        <x:v>76</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>77</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="s">
-        <x:v>78</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+        <x:v>89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="16">
       <x:c r="A10" s="4" t="s">
-        <x:v>79</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>80</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
+        <x:v>91</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="16">
       <x:c r="A11" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>82</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+        <x:v>93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="16">
       <x:c r="A12" s="4" t="s">
-        <x:v>83</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>84</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+        <x:v>95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="16">
       <x:c r="A13" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>86</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
+        <x:v>97</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="16">
       <x:c r="A14" s="4" t="s">
-        <x:v>87</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>88</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
+        <x:v>99</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="16">
       <x:c r="A15" s="4" t="s">
-        <x:v>89</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>90</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="3" t="s">
-        <x:v>91</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
+        <x:v>102</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="32">
       <x:c r="A18" s="4" t="s">
-        <x:v>92</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
+        <x:v>104</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="32">
       <x:c r="A19" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>95</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
+        <x:v>106</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="16">
       <x:c r="A20" s="4" t="s">
-        <x:v>96</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>97</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="4" t="s">
-        <x:v>98</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
-        <x:v>99</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1"/>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="3" t="s">
-        <x:v>100</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="4" t="s">
-        <x:v>101</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1"/>
@@ -3340,78 +3435,78 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultColWidth="14.430000305175781" defaultRowHeight="15"/>
+  <x:sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" customWidth="1"/>
     <x:col min="2" max="2" width="18" customWidth="1"/>
     <x:col min="3" max="3" width="30" customWidth="1"/>
     <x:col min="4" max="4" width="46" customWidth="1"/>
-    <x:col min="5" max="5" width="40" customWidth="1"/>
+    <x:col min="5" max="5" width="55.5" customWidth="1"/>
     <x:col min="6" max="6" width="9" customWidth="1"/>
     <x:col min="7" max="7" width="13" customWidth="1"/>
     <x:col min="8" max="8" width="14" customWidth="1"/>
     <x:col min="9" max="9" width="8" customWidth="1"/>
     <x:col min="10" max="10" width="9" customWidth="1"/>
     <x:col min="11" max="11" width="10" customWidth="1"/>
-    <x:col min="12" max="12" width="24.56999969482422" customWidth="1"/>
+    <x:col min="12" max="12" width="24.5" customWidth="1"/>
     <x:col min="13" max="13" width="11" customWidth="1"/>
     <x:col min="14" max="14" width="16" customWidth="1"/>
     <x:col min="15" max="15" width="10" customWidth="1"/>
     <x:col min="16" max="16" width="20" customWidth="1"/>
-    <x:col min="17" max="26" width="8.710000038146973" customWidth="1"/>
+    <x:col min="17" max="26" width="8.6640625" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="2" t="s">
-        <x:v>103</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>104</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>105</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>106</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>107</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="F1" s="2" t="s">
-        <x:v>108</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="G1" s="2" t="s">
-        <x:v>109</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="H1" s="2" t="s">
-        <x:v>110</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="I1" s="2" t="s">
-        <x:v>111</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="J1" s="2" t="s">
-        <x:v>112</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="K1" s="2" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="L1" s="2" t="s">
-        <x:v>113</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="M1" s="2" t="s">
-        <x:v>114</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="N1" s="2" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="O1" s="2" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="P1" s="2" t="s">
-        <x:v>115</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
+        <x:v>126</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="48" hidden="1">
       <x:c r="A2" s="6" t="str">
         <x:v>KS-T-001</x:v>
       </x:c>
@@ -3443,14 +3538,14 @@
       <x:c r="J2" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K2" s="9" t="str">
+      <x:c r="K2" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L2" s="9" t="str">
+      <x:c r="L2" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M2" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M2" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N2" s="6"/>
       <x:c r="O2" s="6"/>
@@ -3458,7 +3553,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="48" hidden="1">
       <x:c r="A3" s="6" t="str">
         <x:v>KS-T-002</x:v>
       </x:c>
@@ -3490,14 +3585,14 @@
       <x:c r="J3" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K3" s="9" t="str">
+      <x:c r="K3" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L3" s="9" t="str">
+      <x:c r="L3" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M3" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M3" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N3" s="6"/>
       <x:c r="O3" s="6"/>
@@ -3505,7 +3600,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="48" hidden="1">
       <x:c r="A4" s="6" t="str">
         <x:v>KS-T-003</x:v>
       </x:c>
@@ -3537,14 +3632,14 @@
       <x:c r="J4" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K4" s="9" t="str">
+      <x:c r="K4" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L4" s="9" t="str">
+      <x:c r="L4" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M4" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M4" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N4" s="6"/>
       <x:c r="O4" s="6"/>
@@ -3552,7 +3647,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="48" hidden="1">
       <x:c r="A5" s="6" t="str">
         <x:v>KS-T-004</x:v>
       </x:c>
@@ -3584,14 +3679,14 @@
       <x:c r="J5" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K5" s="9" t="str">
+      <x:c r="K5" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L5" s="9" t="str">
+      <x:c r="L5" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M5" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M5" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N5" s="6"/>
       <x:c r="O5" s="6"/>
@@ -3599,7 +3694,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="41.25" customHeight="1">
+    <x:row r="6" ht="41.25" hidden="1" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>KS-T-005</x:v>
       </x:c>
@@ -3633,24 +3728,22 @@
       <x:c r="J6" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K6" s="9" t="str">
-        <x:v>Fail</x:v>
-      </x:c>
-      <x:c r="L6" s="11" t="str">
+      <x:c r="K6" s="6" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L6" s="10" t="str">
         <x:v>Jenny (emulator); Rui / Sam</x:v>
       </x:c>
-      <x:c r="M6" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="N6" s="6" t="str">
-        <x:v>docs/testing-evidence/release-test-round-1/KS-T-005-password-reset-provider-restriction.png</x:v>
-      </x:c>
+      <x:c r="M6" s="11" t="n">
+        <x:v>46284</x:v>
+      </x:c>
+      <x:c r="N6" s="6"/>
       <x:c r="O6" s="6"/>
-      <x:c r="P6" s="12" t="str">
-        <x:v>Tested with emulator, received OTP code in server terminal not the real email. Rui / Sam recorded this case as Fail on 2026-09-19. GitHub defect link pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+      <x:c r="P6" s="7" t="str">
+        <x:v>Retested as Pass in the updated test plan. Historical screenshot removed because it contained personal information. Replacement evidence and retest metadata are pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" hidden="1">
       <x:c r="A7" s="6" t="str">
         <x:v>KS-T-006</x:v>
       </x:c>
@@ -3683,18 +3776,18 @@
       <x:c r="J7" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K7" s="9" t="str">
+      <x:c r="K7" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L7" s="11" t="str">
+      <x:c r="L7" s="10" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="M7" s="14"/>
+      <x:c r="M7" s="11"/>
       <x:c r="N7" s="6"/>
       <x:c r="O7" s="6"/>
       <x:c r="P7" s="7"/>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="48" hidden="1">
       <x:c r="A8" s="6" t="str">
         <x:v>KS-T-007</x:v>
       </x:c>
@@ -3727,18 +3820,18 @@
       <x:c r="J8" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K8" s="9" t="str">
+      <x:c r="K8" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L8" s="11" t="str">
+      <x:c r="L8" s="10" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="M8" s="14"/>
+      <x:c r="M8" s="11"/>
       <x:c r="N8" s="6"/>
       <x:c r="O8" s="6"/>
       <x:c r="P8" s="7"/>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="208" hidden="1">
       <x:c r="A9" s="6" t="str">
         <x:v>KS-T-008</x:v>
       </x:c>
@@ -3770,22 +3863,22 @@
       <x:c r="J9" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K9" s="9" t="str">
+      <x:c r="K9" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L9" s="9" t="str">
+      <x:c r="L9" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="M9" s="14"/>
+      <x:c r="M9" s="11"/>
       <x:c r="N9" s="6"/>
       <x:c r="O9" s="6" t="str">
         <x:v>KS-B-003</x:v>
       </x:c>
-      <x:c r="P9" s="9" t="str">
+      <x:c r="P9" s="6" t="str">
         <x:v>KS-B-003 | KS-T-008 | Profile | Change-password dialog: floating labels overlap the field above (no spacing between the three TextFormFields) | Profile &gt; Change password, observe dialog | S4 Cosmetic | Jenny | Jenny | Open |  | Add SizedBox(height:16) between fields</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="48" hidden="1">
       <x:c r="A10" s="6" t="str">
         <x:v>KS-T-009</x:v>
       </x:c>
@@ -3818,18 +3911,18 @@
       <x:c r="J10" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K10" s="9" t="str">
+      <x:c r="K10" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L10" s="9" t="str">
+      <x:c r="L10" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="M10" s="14"/>
+      <x:c r="M10" s="11"/>
       <x:c r="N10" s="6"/>
       <x:c r="O10" s="6"/>
       <x:c r="P10" s="7"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="48" hidden="1">
       <x:c r="A11" s="6" t="str">
         <x:v>KS-T-010</x:v>
       </x:c>
@@ -3860,14 +3953,14 @@
       <x:c r="J11" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K11" s="9" t="str">
+      <x:c r="K11" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L11" s="9" t="str">
+      <x:c r="L11" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M11" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M11" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N11" s="6"/>
       <x:c r="O11" s="6"/>
@@ -3875,7 +3968,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="32" hidden="1">
       <x:c r="A12" s="6" t="str">
         <x:v>KS-T-011</x:v>
       </x:c>
@@ -3907,18 +4000,18 @@
       <x:c r="J12" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K12" s="9" t="str">
+      <x:c r="K12" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L12" s="9" t="str">
+      <x:c r="L12" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="M12" s="14"/>
+      <x:c r="M12" s="11"/>
       <x:c r="N12" s="6"/>
       <x:c r="O12" s="6"/>
       <x:c r="P12" s="7"/>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="48" hidden="1">
       <x:c r="A13" s="6" t="str">
         <x:v>KS-T-012</x:v>
       </x:c>
@@ -3951,14 +4044,14 @@
       <x:c r="J13" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K13" s="9" t="str">
+      <x:c r="K13" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L13" s="9" t="str">
+      <x:c r="L13" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M13" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M13" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N13" s="6"/>
       <x:c r="O13" s="6"/>
@@ -3966,7 +4059,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="288" hidden="1">
       <x:c r="A14" s="6" t="str">
         <x:v>KS-T-013</x:v>
       </x:c>
@@ -3998,22 +4091,22 @@
       <x:c r="J14" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K14" s="9" t="str">
+      <x:c r="K14" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L14" s="13" t="str">
+      <x:c r="L14" s="9" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="M14" s="14"/>
+      <x:c r="M14" s="11"/>
       <x:c r="N14" s="6"/>
       <x:c r="O14" s="6" t="str">
         <x:v>KS-B-002</x:v>
       </x:c>
-      <x:c r="P14" s="12" t="str">
+      <x:c r="P14" s="7" t="str">
         <x:v>KS-B-002 | KS-T-013 | Profile | Registration accepts displayName &gt;30 chars; edit dialog silently truncates to 30 (inconsistent length limits across entry points) | Register with a 32-char nickname, then edit nickname in Profile and type a 33rd char | S3 Minor | Jenny | Jenny | Open |  | Server /auth/register lacks the 2-30 length check that PUT /users has (users.ts:59); client edit uses maxLength:30</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="64" hidden="1">
       <x:c r="A15" s="6" t="str">
         <x:v>KS-T-014</x:v>
       </x:c>
@@ -4047,11 +4140,11 @@
       <x:c r="K15" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L15" s="9" t="str">
+      <x:c r="L15" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M15" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M15" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N15" s="6"/>
       <x:c r="O15" s="6"/>
@@ -4059,7 +4152,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="48" hidden="1">
       <x:c r="A16" s="6" t="str">
         <x:v>KS-T-015</x:v>
       </x:c>
@@ -4091,14 +4184,14 @@
       <x:c r="J16" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K16" s="9" t="str">
+      <x:c r="K16" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L16" s="9" t="str">
+      <x:c r="L16" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M16" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M16" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N16" s="6"/>
       <x:c r="O16" s="6"/>
@@ -4106,7 +4199,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="48" hidden="1">
       <x:c r="A17" s="6" t="str">
         <x:v>KS-T-016</x:v>
       </x:c>
@@ -4138,14 +4231,14 @@
       <x:c r="J17" s="6" t="str">
         <x:v>Jenny</x:v>
       </x:c>
-      <x:c r="K17" s="9" t="str">
+      <x:c r="K17" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="L17" s="9" t="str">
+      <x:c r="L17" s="6" t="str">
         <x:v>Jenny; Rui / Sam</x:v>
       </x:c>
-      <x:c r="M17" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M17" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N17" s="6"/>
       <x:c r="O17" s="6"/>
@@ -4153,7 +4246,7 @@
         <x:v>Also passed by Rui / Sam on 2026-09-19 (Chinese test plan).</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="64" hidden="1">
       <x:c r="A18" s="6" t="str">
         <x:v>KS-T-017</x:v>
       </x:c>
@@ -4192,8 +4285,8 @@
       <x:c r="L18" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M18" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M18" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N18" s="6"/>
       <x:c r="O18" s="6"/>
@@ -4201,7 +4294,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="32" hidden="1">
       <x:c r="A19" s="6" t="str">
         <x:v>KS-T-018</x:v>
       </x:c>
@@ -4215,7 +4308,7 @@
         <x:v>1. Add 1–5 photos from gallery
 2. Add via camera</x:v>
       </x:c>
-      <x:c r="E19" s="7" t="str">
+      <x:c r="E19" s="19" t="str">
         <x:v>Photos upload, thumbnails shown in step list and on the item</x:v>
       </x:c>
       <x:c r="F19" s="8" t="str">
@@ -4234,15 +4327,17 @@
         <x:v>Jack</x:v>
       </x:c>
       <x:c r="K19" s="6" t="str">
-        <x:v>Not run</x:v>
-      </x:c>
-      <x:c r="L19" s="6"/>
-      <x:c r="M19" s="14"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L19" s="20" t="str">
+        <x:v>Jenny</x:v>
+      </x:c>
+      <x:c r="M19" s="11"/>
       <x:c r="N19" s="6"/>
       <x:c r="O19" s="6"/>
       <x:c r="P19" s="7"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="32" hidden="1">
       <x:c r="A20" s="6" t="str">
         <x:v>KS-T-019</x:v>
       </x:c>
@@ -4275,15 +4370,15 @@
         <x:v>Jack</x:v>
       </x:c>
       <x:c r="K20" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L20" s="6"/>
-      <x:c r="M20" s="14"/>
+      <x:c r="M20" s="11"/>
       <x:c r="N20" s="6"/>
       <x:c r="O20" s="6"/>
       <x:c r="P20" s="7"/>
     </x:row>
-    <x:row r="21" ht="15.75" customHeight="1">
+    <x:row r="21" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A21" s="6" t="str">
         <x:v>KS-T-020</x:v>
       </x:c>
@@ -4322,8 +4417,8 @@
       <x:c r="L21" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M21" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M21" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N21" s="6"/>
       <x:c r="O21" s="6"/>
@@ -4331,7 +4426,7 @@
         <x:v>Marked Fail by Rui / Sam on 2026-09-19; GitHub defect link pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15.75" customHeight="1">
+    <x:row r="22" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A22" s="6" t="str">
         <x:v>KS-T-021</x:v>
       </x:c>
@@ -4368,8 +4463,8 @@
       <x:c r="L22" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M22" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M22" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N22" s="6"/>
       <x:c r="O22" s="6"/>
@@ -4377,7 +4472,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="15.75" customHeight="1">
+    <x:row r="23" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A23" s="6" t="str">
         <x:v>KS-T-022</x:v>
       </x:c>
@@ -4387,7 +4482,7 @@
       <x:c r="C23" s="7" t="str">
         <x:v>GPS location on publish</x:v>
       </x:c>
-      <x:c r="D23" s="7" t="str">
+      <x:c r="D23" s="19" t="str">
         <x:v>1. Grant location permission
 2. Publish with current location
 3. Deny permission and publish</x:v>
@@ -4411,15 +4506,17 @@
         <x:v>Jack</x:v>
       </x:c>
       <x:c r="K23" s="6" t="str">
-        <x:v>Not run</x:v>
-      </x:c>
-      <x:c r="L23" s="6"/>
-      <x:c r="M23" s="14"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L23" s="20" t="str">
+        <x:v>Jenny</x:v>
+      </x:c>
+      <x:c r="M23" s="11"/>
       <x:c r="N23" s="6"/>
       <x:c r="O23" s="6"/>
       <x:c r="P23" s="7"/>
     </x:row>
-    <x:row r="24" ht="15.75" customHeight="1">
+    <x:row r="24" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A24" s="6" t="str">
         <x:v>KS-T-023</x:v>
       </x:c>
@@ -4458,8 +4555,8 @@
       <x:c r="L24" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M24" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M24" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N24" s="6"/>
       <x:c r="O24" s="6"/>
@@ -4467,7 +4564,7 @@
         <x:v>Marked Fail by Rui / Sam on 2026-09-19; GitHub defect link pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="15.75" customHeight="1">
+    <x:row r="25" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A25" s="6" t="str">
         <x:v>KS-T-024</x:v>
       </x:c>
@@ -4505,8 +4602,8 @@
       <x:c r="L25" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M25" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M25" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N25" s="6"/>
       <x:c r="O25" s="6"/>
@@ -4514,7 +4611,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="15.75" customHeight="1">
+    <x:row r="26" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A26" s="6" t="str">
         <x:v>KS-T-025</x:v>
       </x:c>
@@ -4551,8 +4648,8 @@
       <x:c r="L26" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M26" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M26" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N26" s="6"/>
       <x:c r="O26" s="6"/>
@@ -4560,7 +4657,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="15.75" customHeight="1">
+    <x:row r="27" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A27" s="6" t="str">
         <x:v>KS-T-026</x:v>
       </x:c>
@@ -4598,8 +4695,8 @@
       <x:c r="L27" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M27" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M27" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N27" s="6"/>
       <x:c r="O27" s="6"/>
@@ -4607,7 +4704,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15.75" customHeight="1">
+    <x:row r="28" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A28" s="6" t="str">
         <x:v>KS-T-027</x:v>
       </x:c>
@@ -4639,10 +4736,12 @@
         <x:v>Rui</x:v>
       </x:c>
       <x:c r="K28" s="6" t="str">
-        <x:v>Not run</x:v>
-      </x:c>
-      <x:c r="L28" s="6"/>
-      <x:c r="M28" s="14"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L28" s="20" t="str">
+        <x:v>Jenny</x:v>
+      </x:c>
+      <x:c r="M28" s="11"/>
       <x:c r="N28" s="6"/>
       <x:c r="O28" s="6"/>
       <x:c r="P28" s="7"/>
@@ -4682,12 +4781,12 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L29" s="6"/>
-      <x:c r="M29" s="14"/>
+      <x:c r="M29" s="11"/>
       <x:c r="N29" s="6"/>
       <x:c r="O29" s="6"/>
       <x:c r="P29" s="7"/>
     </x:row>
-    <x:row r="30" ht="15.75" customHeight="1">
+    <x:row r="30" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A30" s="6" t="str">
         <x:v>KS-T-029</x:v>
       </x:c>
@@ -4720,15 +4819,15 @@
         <x:v>Rui</x:v>
       </x:c>
       <x:c r="K30" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L30" s="6"/>
-      <x:c r="M30" s="14"/>
+      <x:c r="M30" s="11"/>
       <x:c r="N30" s="6"/>
       <x:c r="O30" s="6"/>
       <x:c r="P30" s="7"/>
     </x:row>
-    <x:row r="31" ht="15.75" customHeight="1">
+    <x:row r="31" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A31" s="6" t="str">
         <x:v>KS-T-030</x:v>
       </x:c>
@@ -4765,8 +4864,8 @@
       <x:c r="L31" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M31" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M31" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N31" s="6"/>
       <x:c r="O31" s="6"/>
@@ -4774,7 +4873,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="15.75" customHeight="1">
+    <x:row r="32" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A32" s="6" t="str">
         <x:v>KS-T-031</x:v>
       </x:c>
@@ -4812,8 +4911,8 @@
       <x:c r="L32" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M32" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M32" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N32" s="6"/>
       <x:c r="O32" s="6"/>
@@ -4821,7 +4920,7 @@
         <x:v>Marked Fail by Rui / Sam on 2026-09-19; GitHub defect link pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="15.75" customHeight="1">
+    <x:row r="33" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A33" s="6" t="str">
         <x:v>KS-T-032</x:v>
       </x:c>
@@ -4860,8 +4959,8 @@
       <x:c r="L33" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M33" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M33" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N33" s="6"/>
       <x:c r="O33" s="6"/>
@@ -4907,12 +5006,12 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L34" s="6"/>
-      <x:c r="M34" s="14"/>
+      <x:c r="M34" s="11"/>
       <x:c r="N34" s="6"/>
       <x:c r="O34" s="6"/>
       <x:c r="P34" s="7"/>
     </x:row>
-    <x:row r="35" ht="15.75" customHeight="1">
+    <x:row r="35" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A35" s="6" t="str">
         <x:v>KS-T-034</x:v>
       </x:c>
@@ -4945,10 +5044,10 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="K35" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L35" s="6"/>
-      <x:c r="M35" s="14"/>
+      <x:c r="M35" s="11"/>
       <x:c r="N35" s="6"/>
       <x:c r="O35" s="6"/>
       <x:c r="P35" s="7"/>
@@ -4963,7 +5062,7 @@
       <x:c r="C36" s="7" t="str">
         <x:v>Notification routing</x:v>
       </x:c>
-      <x:c r="D36" s="7" t="str">
+      <x:c r="D36" s="19" t="str">
         <x:v>Setup: two devices; B sends A a message while A is backgrounded
 1. Wait for push on A's device
 2. Tap the notification</x:v>
@@ -4990,12 +5089,12 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L36" s="6"/>
-      <x:c r="M36" s="14"/>
+      <x:c r="M36" s="11"/>
       <x:c r="N36" s="6"/>
       <x:c r="O36" s="6"/>
       <x:c r="P36" s="7"/>
     </x:row>
-    <x:row r="37" ht="15.75" customHeight="1">
+    <x:row r="37" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A37" s="6" t="str">
         <x:v>KS-T-036</x:v>
       </x:c>
@@ -5034,8 +5133,8 @@
       <x:c r="L37" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M37" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M37" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N37" s="6"/>
       <x:c r="O37" s="6"/>
@@ -5043,7 +5142,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="15.75" customHeight="1">
+    <x:row r="38" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A38" s="6" t="str">
         <x:v>KS-T-037</x:v>
       </x:c>
@@ -5076,15 +5175,15 @@
         <x:v>Jaeger</x:v>
       </x:c>
       <x:c r="K38" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L38" s="6"/>
-      <x:c r="M38" s="14"/>
+      <x:c r="M38" s="11"/>
       <x:c r="N38" s="6"/>
       <x:c r="O38" s="6"/>
       <x:c r="P38" s="7"/>
     </x:row>
-    <x:row r="39" ht="15.75" customHeight="1">
+    <x:row r="39" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A39" s="6" t="str">
         <x:v>KS-T-038</x:v>
       </x:c>
@@ -5122,8 +5221,8 @@
       <x:c r="L39" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M39" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M39" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N39" s="6"/>
       <x:c r="O39" s="6"/>
@@ -5131,7 +5230,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="15.75" customHeight="1">
+    <x:row r="40" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A40" s="6" t="str">
         <x:v>KS-T-039</x:v>
       </x:c>
@@ -5164,15 +5263,15 @@
         <x:v>Jaeger</x:v>
       </x:c>
       <x:c r="K40" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L40" s="6"/>
-      <x:c r="M40" s="14"/>
+      <x:c r="M40" s="11"/>
       <x:c r="N40" s="6"/>
       <x:c r="O40" s="6"/>
       <x:c r="P40" s="7"/>
     </x:row>
-    <x:row r="41" ht="15.75" customHeight="1">
+    <x:row r="41" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A41" s="6" t="str">
         <x:v>KS-T-040</x:v>
       </x:c>
@@ -5205,15 +5304,15 @@
         <x:v>Jaeger</x:v>
       </x:c>
       <x:c r="K41" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L41" s="6"/>
-      <x:c r="M41" s="14"/>
+      <x:c r="M41" s="11"/>
       <x:c r="N41" s="6"/>
       <x:c r="O41" s="6"/>
       <x:c r="P41" s="7"/>
     </x:row>
-    <x:row r="42" ht="15.75" customHeight="1">
+    <x:row r="42" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A42" s="6" t="str">
         <x:v>KS-T-041</x:v>
       </x:c>
@@ -5245,15 +5344,15 @@
         <x:v>Jaeger</x:v>
       </x:c>
       <x:c r="K42" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L42" s="6"/>
-      <x:c r="M42" s="14"/>
+      <x:c r="M42" s="11"/>
       <x:c r="N42" s="6"/>
       <x:c r="O42" s="6"/>
       <x:c r="P42" s="7"/>
     </x:row>
-    <x:row r="43" ht="15.75" customHeight="1">
+    <x:row r="43" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A43" s="6" t="str">
         <x:v>KS-T-042</x:v>
       </x:c>
@@ -5263,7 +5362,7 @@
       <x:c r="C43" s="7" t="str">
         <x:v>Swipe delete conversation</x:v>
       </x:c>
-      <x:c r="D43" s="7" t="str">
+      <x:c r="D43" s="19" t="str">
         <x:v>1. Swipe a conversation
 2. Confirm</x:v>
       </x:c>
@@ -5286,15 +5385,15 @@
         <x:v>Jaeger</x:v>
       </x:c>
       <x:c r="K43" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L43" s="6"/>
-      <x:c r="M43" s="14"/>
+      <x:c r="M43" s="11"/>
       <x:c r="N43" s="6"/>
       <x:c r="O43" s="6"/>
       <x:c r="P43" s="7"/>
     </x:row>
-    <x:row r="44" ht="15.75" customHeight="1">
+    <x:row r="44" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A44" s="6" t="str">
         <x:v>KS-T-043</x:v>
       </x:c>
@@ -5327,10 +5426,10 @@
         <x:v>Jack</x:v>
       </x:c>
       <x:c r="K44" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L44" s="6"/>
-      <x:c r="M44" s="14"/>
+      <x:c r="M44" s="11"/>
       <x:c r="N44" s="6"/>
       <x:c r="O44" s="6"/>
       <x:c r="P44" s="7"/>
@@ -5370,7 +5469,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L45" s="6"/>
-      <x:c r="M45" s="14"/>
+      <x:c r="M45" s="11"/>
       <x:c r="N45" s="6"/>
       <x:c r="O45" s="6"/>
       <x:c r="P45" s="7"/>
@@ -5410,7 +5509,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L46" s="6"/>
-      <x:c r="M46" s="14"/>
+      <x:c r="M46" s="11"/>
       <x:c r="N46" s="6"/>
       <x:c r="O46" s="6"/>
       <x:c r="P46" s="7"/>
@@ -5450,13 +5549,13 @@
       <x:c r="K47" s="6" t="str">
         <x:v>Not run</x:v>
       </x:c>
-      <x:c r="L47" s="6"/>
-      <x:c r="M47" s="14"/>
+      <x:c r="L47" s="20"/>
+      <x:c r="M47" s="11"/>
       <x:c r="N47" s="6"/>
       <x:c r="O47" s="6"/>
       <x:c r="P47" s="7"/>
     </x:row>
-    <x:row r="48" ht="15.75" customHeight="1">
+    <x:row r="48" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A48" s="6" t="str">
         <x:v>KS-T-047</x:v>
       </x:c>
@@ -5493,8 +5592,8 @@
       <x:c r="L48" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M48" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M48" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N48" s="6"/>
       <x:c r="O48" s="6"/>
@@ -5502,7 +5601,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="15.75" customHeight="1">
+    <x:row r="49" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A49" s="6" t="str">
         <x:v>KS-T-048</x:v>
       </x:c>
@@ -5539,8 +5638,8 @@
       <x:c r="L49" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M49" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M49" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N49" s="6"/>
       <x:c r="O49" s="6"/>
@@ -5548,7 +5647,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="15.75" customHeight="1">
+    <x:row r="50" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A50" s="6" t="str">
         <x:v>KS-T-049</x:v>
       </x:c>
@@ -5585,8 +5684,8 @@
       <x:c r="L50" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M50" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M50" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N50" s="6"/>
       <x:c r="O50" s="6"/>
@@ -5594,7 +5693,7 @@
         <x:v>Imported from the Chinese test plan completed by Rui / Sam on 2026-09-19.</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="15.75" customHeight="1">
+    <x:row r="51" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A51" s="6" t="str">
         <x:v>KS-T-050</x:v>
       </x:c>
@@ -5626,11 +5725,11 @@
       <x:c r="J51" s="6" t="str">
         <x:v>Sam</x:v>
       </x:c>
-      <x:c r="K51" s="9" t="str">
+      <x:c r="K51" s="6" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="L51" s="6"/>
-      <x:c r="M51" s="14"/>
+      <x:c r="M51" s="11"/>
       <x:c r="N51" s="6"/>
       <x:c r="O51" s="6"/>
       <x:c r="P51" s="7"/>
@@ -5670,7 +5769,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L52" s="6"/>
-      <x:c r="M52" s="14"/>
+      <x:c r="M52" s="11"/>
       <x:c r="N52" s="6"/>
       <x:c r="O52" s="6"/>
       <x:c r="P52" s="7"/>
@@ -5710,12 +5809,12 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L53" s="6"/>
-      <x:c r="M53" s="14"/>
+      <x:c r="M53" s="11"/>
       <x:c r="N53" s="6"/>
       <x:c r="O53" s="6"/>
       <x:c r="P53" s="7"/>
     </x:row>
-    <x:row r="54" ht="15.75" customHeight="1">
+    <x:row r="54" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A54" s="6" t="str">
         <x:v>KS-T-053</x:v>
       </x:c>
@@ -5748,10 +5847,10 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="K54" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L54" s="6"/>
-      <x:c r="M54" s="14"/>
+      <x:c r="M54" s="11"/>
       <x:c r="N54" s="6"/>
       <x:c r="O54" s="6"/>
       <x:c r="P54" s="7"/>
@@ -5766,7 +5865,7 @@
       <x:c r="C55" s="7" t="str">
         <x:v>App cold start time</x:v>
       </x:c>
-      <x:c r="D55" s="7" t="str">
+      <x:c r="D55" s="19" t="str">
         <x:v>1. Force-kill the app
 2. Cold start on emulator and real device, timing tap-to-home-interactive
 3. Repeat 3x per device</x:v>
@@ -5793,7 +5892,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L55" s="6"/>
-      <x:c r="M55" s="14"/>
+      <x:c r="M55" s="11"/>
       <x:c r="N55" s="6"/>
       <x:c r="O55" s="6"/>
       <x:c r="P55" s="7"/>
@@ -5808,7 +5907,7 @@
       <x:c r="C56" s="7" t="str">
         <x:v>Home feed full-scroll smoothness</x:v>
       </x:c>
-      <x:c r="D56" s="7" t="str">
+      <x:c r="D56" s="19" t="str">
         <x:v>1. Seed 50+ items (Test Data sheet)
 2. Scroll the entire home feed on emulator and real device
 3. Note any jank / freezes</x:v>
@@ -5835,7 +5934,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L56" s="6"/>
-      <x:c r="M56" s="14"/>
+      <x:c r="M56" s="11"/>
       <x:c r="N56" s="6"/>
       <x:c r="O56" s="6"/>
       <x:c r="P56" s="7"/>
@@ -5850,7 +5949,7 @@
       <x:c r="C57" s="7" t="str">
         <x:v>API latency baseline &amp; light load</x:v>
       </x:c>
-      <x:c r="D57" s="7" t="str">
+      <x:c r="D57" s="19" t="str">
         <x:v>1. Measure response time of key GET endpoints (items list, item detail, chat history)
 2. Load one endpoint with ~20 concurrent requests for 30 s (autocannon/k6/hey)
 3. Record p50/p95 and error count</x:v>
@@ -5877,12 +5976,12 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L57" s="6"/>
-      <x:c r="M57" s="14"/>
+      <x:c r="M57" s="11"/>
       <x:c r="N57" s="6"/>
       <x:c r="O57" s="6"/>
       <x:c r="P57" s="7"/>
     </x:row>
-    <x:row r="58" ht="15.75" customHeight="1">
+    <x:row r="58" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A58" s="6" t="str">
         <x:v>KS-T-057</x:v>
       </x:c>
@@ -5892,7 +5991,7 @@
       <x:c r="C58" s="7" t="str">
         <x:v>Item detail image loading</x:v>
       </x:c>
-      <x:c r="D58" s="7" t="str">
+      <x:c r="D58" s="19" t="str">
         <x:v>1. Open a 5-photo item on a real device
 2. Repeat on a throttled connection if possible</x:v>
       </x:c>
@@ -5915,15 +6014,15 @@
         <x:v>Jack</x:v>
       </x:c>
       <x:c r="K58" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L58" s="6"/>
-      <x:c r="M58" s="14"/>
+      <x:c r="M58" s="11"/>
       <x:c r="N58" s="6"/>
       <x:c r="O58" s="6"/>
       <x:c r="P58" s="7"/>
     </x:row>
-    <x:row r="59" ht="15.75" customHeight="1">
+    <x:row r="59" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A59" s="6" t="str">
         <x:v>KS-T-058</x:v>
       </x:c>
@@ -5956,15 +6055,15 @@
         <x:v>Jenny</x:v>
       </x:c>
       <x:c r="K59" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L59" s="6"/>
-      <x:c r="M59" s="14"/>
+      <x:c r="M59" s="11"/>
       <x:c r="N59" s="6"/>
       <x:c r="O59" s="6"/>
       <x:c r="P59" s="7"/>
     </x:row>
-    <x:row r="60" ht="15.75" customHeight="1">
+    <x:row r="60" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A60" s="6" t="str">
         <x:v>KS-T-059</x:v>
       </x:c>
@@ -5996,15 +6095,15 @@
         <x:v>Jack</x:v>
       </x:c>
       <x:c r="K60" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L60" s="6"/>
-      <x:c r="M60" s="14"/>
+      <x:c r="M60" s="11"/>
       <x:c r="N60" s="6"/>
       <x:c r="O60" s="6"/>
       <x:c r="P60" s="7"/>
     </x:row>
-    <x:row r="61" ht="15.75" customHeight="1">
+    <x:row r="61" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A61" s="6" t="str">
         <x:v>KS-T-060</x:v>
       </x:c>
@@ -6041,8 +6140,8 @@
       <x:c r="L61" s="6" t="str">
         <x:v>Rui / Sam</x:v>
       </x:c>
-      <x:c r="M61" s="14" t="d">
-        <x:v>2026-09-19T00:00:00.000Z</x:v>
+      <x:c r="M61" s="11" t="n">
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="N61" s="6"/>
       <x:c r="O61" s="6"/>
@@ -6050,7 +6149,7 @@
         <x:v>Marked Fail by Rui / Sam on 2026-09-19; GitHub defect link pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="15.75" customHeight="1">
+    <x:row r="62" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A62" s="6" t="str">
         <x:v>KS-T-061</x:v>
       </x:c>
@@ -6082,15 +6181,15 @@
         <x:v>Jaeger</x:v>
       </x:c>
       <x:c r="K62" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L62" s="6"/>
-      <x:c r="M62" s="14"/>
+      <x:c r="M62" s="11"/>
       <x:c r="N62" s="6"/>
       <x:c r="O62" s="6"/>
       <x:c r="P62" s="7"/>
     </x:row>
-    <x:row r="63" ht="15.75" customHeight="1">
+    <x:row r="63" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A63" s="6" t="str">
         <x:v>KS-T-062</x:v>
       </x:c>
@@ -6122,15 +6221,15 @@
         <x:v>Rui</x:v>
       </x:c>
       <x:c r="K63" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L63" s="6"/>
-      <x:c r="M63" s="14"/>
+      <x:c r="M63" s="11"/>
       <x:c r="N63" s="6"/>
       <x:c r="O63" s="6"/>
       <x:c r="P63" s="7"/>
     </x:row>
-    <x:row r="64" ht="15.75" customHeight="1">
+    <x:row r="64" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A64" s="6" t="str">
         <x:v>KS-T-063</x:v>
       </x:c>
@@ -6140,7 +6239,7 @@
       <x:c r="C64" s="7" t="str">
         <x:v>App resume / background</x:v>
       </x:c>
-      <x:c r="D64" s="7" t="str">
+      <x:c r="D64" s="19" t="str">
         <x:v>1. Background app mid-flow
 2. Return after 1 min and 10 min</x:v>
       </x:c>
@@ -6163,15 +6262,15 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="K64" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L64" s="6"/>
-      <x:c r="M64" s="14"/>
+      <x:c r="M64" s="11"/>
       <x:c r="N64" s="6"/>
       <x:c r="O64" s="6"/>
       <x:c r="P64" s="7"/>
     </x:row>
-    <x:row r="65" ht="15.75" customHeight="1">
+    <x:row r="65" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A65" s="6" t="str">
         <x:v>KS-T-064</x:v>
       </x:c>
@@ -6204,15 +6303,15 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="K65" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L65" s="6"/>
-      <x:c r="M65" s="14"/>
+      <x:c r="M65" s="11"/>
       <x:c r="N65" s="6"/>
       <x:c r="O65" s="6"/>
       <x:c r="P65" s="7"/>
     </x:row>
-    <x:row r="66" ht="15.75" customHeight="1">
+    <x:row r="66" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A66" s="6" t="str">
         <x:v>KS-T-065</x:v>
       </x:c>
@@ -6246,10 +6345,10 @@
         <x:v>Jenny</x:v>
       </x:c>
       <x:c r="K66" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L66" s="6"/>
-      <x:c r="M66" s="14"/>
+      <x:c r="M66" s="11"/>
       <x:c r="N66" s="6"/>
       <x:c r="O66" s="6"/>
       <x:c r="P66" s="7"/>
@@ -6291,7 +6390,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L67" s="6"/>
-      <x:c r="M67" s="14"/>
+      <x:c r="M67" s="11"/>
       <x:c r="N67" s="6"/>
       <x:c r="O67" s="6"/>
       <x:c r="P67" s="7"/>
@@ -6333,7 +6432,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L68" s="6"/>
-      <x:c r="M68" s="14"/>
+      <x:c r="M68" s="11"/>
       <x:c r="N68" s="6"/>
       <x:c r="O68" s="6"/>
       <x:c r="P68" s="7"/>
@@ -6375,7 +6474,7 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L69" s="6"/>
-      <x:c r="M69" s="14"/>
+      <x:c r="M69" s="11"/>
       <x:c r="N69" s="6"/>
       <x:c r="O69" s="6"/>
       <x:c r="P69" s="7"/>
@@ -6417,12 +6516,12 @@
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="L70" s="6"/>
-      <x:c r="M70" s="14"/>
+      <x:c r="M70" s="11"/>
       <x:c r="N70" s="6"/>
       <x:c r="O70" s="6"/>
       <x:c r="P70" s="7"/>
     </x:row>
-    <x:row r="71" ht="15.75" customHeight="1">
+    <x:row r="71" ht="15.75" hidden="1" customHeight="1">
       <x:c r="A71" s="6" t="str">
         <x:v>KS-T-070</x:v>
       </x:c>
@@ -6455,10 +6554,10 @@
         <x:v>Rui</x:v>
       </x:c>
       <x:c r="K71" s="6" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="L71" s="6"/>
-      <x:c r="M71" s="14"/>
+      <x:c r="M71" s="11"/>
       <x:c r="N71" s="6"/>
       <x:c r="O71" s="6"/>
       <x:c r="P71" s="7"/>
@@ -7394,22 +7493,16 @@
     <x:row r="1000" ht="15.75" customHeight="1"/>
   </x:sheetData>
   <x:conditionalFormatting sqref="K2:K71">
-    <x:cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <x:formula>"Pass"</x:formula>
     </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="K2:K71">
-    <x:cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <x:formula>"Fail"</x:formula>
     </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="K2:K71">
-    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <x:cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <x:formula>"Blocked"</x:formula>
     </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="K2:K71">
-    <x:cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+    <x:cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
       <x:formula>"Not run"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -7424,7 +7517,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultColWidth="14.430000305175781" defaultRowHeight="15"/>
+  <x:sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11" customWidth="1"/>
     <x:col min="2" max="2" width="12" customWidth="1"/>
@@ -7434,930 +7527,930 @@
     <x:col min="6" max="6" width="10" customWidth="1"/>
     <x:col min="7" max="10" width="11" customWidth="1"/>
     <x:col min="11" max="11" width="24" customWidth="1"/>
-    <x:col min="12" max="26" width="8.710000038146973" customWidth="1"/>
+    <x:col min="12" max="26" width="8.6640625" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="2" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>116</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>104</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>117</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>118</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="F1" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="G1" s="2" t="s">
-        <x:v>120</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="H1" s="2" t="s">
-        <x:v>121</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="I1" s="2" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J1" s="2" t="s">
-        <x:v>114</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="K1" s="2" t="s">
-        <x:v>115</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
+        <x:v>126</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="48">
       <x:c r="A2" s="7" t="s">
-        <x:v>122</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B2" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C2" s="7" t="s">
-        <x:v>124</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="D2" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E2" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="F2" s="7" t="s">
-        <x:v>127</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="G2" s="7" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="H2" s="7" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I2" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="J2" s="7"/>
       <x:c r="K2" s="7" t="s">
-        <x:v>129</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="19" t="str">
-        <x:v>KS-B-002</x:v>
-      </x:c>
-      <x:c r="B3" s="19" t="str">
-        <x:v>KS-T-013</x:v>
-      </x:c>
-      <x:c r="C3" s="19" t="str">
-        <x:v>Profile</x:v>
-      </x:c>
-      <x:c r="D3" s="19" t="str">
-        <x:v>Registration accepted display names longer than 30 characters while Profile editing capped them at 30.</x:v>
-      </x:c>
-      <x:c r="E3" s="19" t="str">
-        <x:v>Register with a 32-character nickname, then edit the nickname in Profile and enter a 33rd character.</x:v>
-      </x:c>
-      <x:c r="F3" s="20" t="str">
-        <x:v>S3 Minor</x:v>
-      </x:c>
-      <x:c r="G3" s="19" t="str">
-        <x:v>Jenny</x:v>
-      </x:c>
-      <x:c r="H3" s="19" t="str">
-        <x:v>Jenny</x:v>
-      </x:c>
-      <x:c r="I3" s="20" t="str">
-        <x:v>Closed</x:v>
-      </x:c>
-      <x:c r="J3" s="21" t="d">
-        <x:v>2026-09-16T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="K3" s="19" t="str">
-        <x:v>Fixed in PR #309 by applying the 2-30 character limit consistently; the linked test case now passes.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="19" t="str">
-        <x:v>KS-B-003</x:v>
-      </x:c>
-      <x:c r="B4" s="19" t="str">
-        <x:v>KS-T-008</x:v>
-      </x:c>
-      <x:c r="C4" s="19" t="str">
-        <x:v>Profile</x:v>
-      </x:c>
-      <x:c r="D4" s="19" t="str">
-        <x:v>Floating labels overlapped adjacent fields in the change-password dialog.</x:v>
-      </x:c>
-      <x:c r="E4" s="19" t="str">
-        <x:v>Open Profile &gt; Change password and inspect spacing between the three password fields.</x:v>
-      </x:c>
-      <x:c r="F4" s="20" t="str">
-        <x:v>S4 Cosmetic</x:v>
-      </x:c>
-      <x:c r="G4" s="19" t="str">
-        <x:v>Jenny</x:v>
-      </x:c>
-      <x:c r="H4" s="19" t="str">
-        <x:v>Jenny</x:v>
-      </x:c>
-      <x:c r="I4" s="20" t="str">
-        <x:v>Closed</x:v>
-      </x:c>
-      <x:c r="J4" s="21" t="d">
-        <x:v>2026-09-16T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="K4" s="19" t="str">
-        <x:v>Fixed in PR #309 by restoring spacing between fields; the linked test case now passes.</x:v>
+        <x:v>140</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="64">
+      <x:c r="A3" s="12" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="I3" s="13" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="J3" s="14">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="K3" s="12" t="s">
+        <x:v>147</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48">
+      <x:c r="A4" s="12" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="H4" s="12" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="J4" s="14">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="K4" s="12" t="s">
+        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="F5" s="10"/>
-      <x:c r="I5" s="10"/>
+      <x:c r="F5" s="9"/>
+      <x:c r="I5" s="9"/>
     </x:row>
     <x:row r="6">
-      <x:c r="F6" s="10"/>
-      <x:c r="I6" s="10"/>
+      <x:c r="F6" s="9"/>
+      <x:c r="I6" s="9"/>
     </x:row>
     <x:row r="7">
-      <x:c r="F7" s="10"/>
-      <x:c r="I7" s="10"/>
+      <x:c r="F7" s="9"/>
+      <x:c r="I7" s="9"/>
     </x:row>
     <x:row r="8">
-      <x:c r="F8" s="10"/>
-      <x:c r="I8" s="10"/>
+      <x:c r="F8" s="9"/>
+      <x:c r="I8" s="9"/>
     </x:row>
     <x:row r="9">
-      <x:c r="F9" s="10"/>
-      <x:c r="I9" s="10"/>
+      <x:c r="F9" s="9"/>
+      <x:c r="I9" s="9"/>
     </x:row>
     <x:row r="10">
-      <x:c r="F10" s="10"/>
-      <x:c r="I10" s="10"/>
+      <x:c r="F10" s="9"/>
+      <x:c r="I10" s="9"/>
     </x:row>
     <x:row r="11">
-      <x:c r="F11" s="10"/>
-      <x:c r="I11" s="10"/>
+      <x:c r="F11" s="9"/>
+      <x:c r="I11" s="9"/>
     </x:row>
     <x:row r="12">
-      <x:c r="F12" s="10"/>
-      <x:c r="I12" s="10"/>
+      <x:c r="F12" s="9"/>
+      <x:c r="I12" s="9"/>
     </x:row>
     <x:row r="13">
-      <x:c r="F13" s="10"/>
-      <x:c r="I13" s="10"/>
+      <x:c r="F13" s="9"/>
+      <x:c r="I13" s="9"/>
     </x:row>
     <x:row r="14">
-      <x:c r="F14" s="10"/>
-      <x:c r="I14" s="10"/>
+      <x:c r="F14" s="9"/>
+      <x:c r="I14" s="9"/>
     </x:row>
     <x:row r="15">
-      <x:c r="F15" s="10"/>
-      <x:c r="I15" s="10"/>
+      <x:c r="F15" s="9"/>
+      <x:c r="I15" s="9"/>
     </x:row>
     <x:row r="16">
-      <x:c r="F16" s="10"/>
-      <x:c r="I16" s="10"/>
+      <x:c r="F16" s="9"/>
+      <x:c r="I16" s="9"/>
     </x:row>
     <x:row r="17">
-      <x:c r="F17" s="10"/>
-      <x:c r="I17" s="10"/>
+      <x:c r="F17" s="9"/>
+      <x:c r="I17" s="9"/>
     </x:row>
     <x:row r="18">
-      <x:c r="F18" s="10"/>
-      <x:c r="I18" s="10"/>
+      <x:c r="F18" s="9"/>
+      <x:c r="I18" s="9"/>
     </x:row>
     <x:row r="19">
-      <x:c r="F19" s="10"/>
-      <x:c r="I19" s="10"/>
+      <x:c r="F19" s="9"/>
+      <x:c r="I19" s="9"/>
     </x:row>
     <x:row r="20">
-      <x:c r="F20" s="10"/>
-      <x:c r="I20" s="10"/>
+      <x:c r="F20" s="9"/>
+      <x:c r="I20" s="9"/>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
-      <x:c r="F21" s="10"/>
-      <x:c r="I21" s="10"/>
+      <x:c r="F21" s="9"/>
+      <x:c r="I21" s="9"/>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
-      <x:c r="F22" s="10"/>
-      <x:c r="I22" s="10"/>
+      <x:c r="F22" s="9"/>
+      <x:c r="I22" s="9"/>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
-      <x:c r="F23" s="10"/>
-      <x:c r="I23" s="10"/>
+      <x:c r="F23" s="9"/>
+      <x:c r="I23" s="9"/>
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
-      <x:c r="F24" s="10"/>
-      <x:c r="I24" s="10"/>
+      <x:c r="F24" s="9"/>
+      <x:c r="I24" s="9"/>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
-      <x:c r="F25" s="10"/>
-      <x:c r="I25" s="10"/>
+      <x:c r="F25" s="9"/>
+      <x:c r="I25" s="9"/>
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1">
-      <x:c r="F26" s="10"/>
-      <x:c r="I26" s="10"/>
+      <x:c r="F26" s="9"/>
+      <x:c r="I26" s="9"/>
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
-      <x:c r="F27" s="10"/>
-      <x:c r="I27" s="10"/>
+      <x:c r="F27" s="9"/>
+      <x:c r="I27" s="9"/>
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
-      <x:c r="F28" s="10"/>
-      <x:c r="I28" s="10"/>
+      <x:c r="F28" s="9"/>
+      <x:c r="I28" s="9"/>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
-      <x:c r="F29" s="10"/>
-      <x:c r="I29" s="10"/>
+      <x:c r="F29" s="9"/>
+      <x:c r="I29" s="9"/>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
-      <x:c r="F30" s="10"/>
-      <x:c r="I30" s="10"/>
+      <x:c r="F30" s="9"/>
+      <x:c r="I30" s="9"/>
     </x:row>
     <x:row r="31" ht="15.75" customHeight="1">
-      <x:c r="F31" s="10"/>
-      <x:c r="I31" s="10"/>
+      <x:c r="F31" s="9"/>
+      <x:c r="I31" s="9"/>
     </x:row>
     <x:row r="32" ht="15.75" customHeight="1">
-      <x:c r="F32" s="10"/>
-      <x:c r="I32" s="10"/>
+      <x:c r="F32" s="9"/>
+      <x:c r="I32" s="9"/>
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1">
-      <x:c r="F33" s="10"/>
-      <x:c r="I33" s="10"/>
+      <x:c r="F33" s="9"/>
+      <x:c r="I33" s="9"/>
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1">
-      <x:c r="F34" s="10"/>
-      <x:c r="I34" s="10"/>
+      <x:c r="F34" s="9"/>
+      <x:c r="I34" s="9"/>
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
-      <x:c r="F35" s="10"/>
-      <x:c r="I35" s="10"/>
+      <x:c r="F35" s="9"/>
+      <x:c r="I35" s="9"/>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
-      <x:c r="F36" s="10"/>
-      <x:c r="I36" s="10"/>
+      <x:c r="F36" s="9"/>
+      <x:c r="I36" s="9"/>
     </x:row>
     <x:row r="37" ht="15.75" customHeight="1">
-      <x:c r="F37" s="10"/>
-      <x:c r="I37" s="10"/>
+      <x:c r="F37" s="9"/>
+      <x:c r="I37" s="9"/>
     </x:row>
     <x:row r="38" ht="15.75" customHeight="1">
-      <x:c r="F38" s="10"/>
-      <x:c r="I38" s="10"/>
+      <x:c r="F38" s="9"/>
+      <x:c r="I38" s="9"/>
     </x:row>
     <x:row r="39" ht="15.75" customHeight="1">
-      <x:c r="F39" s="10"/>
-      <x:c r="I39" s="10"/>
+      <x:c r="F39" s="9"/>
+      <x:c r="I39" s="9"/>
     </x:row>
     <x:row r="40" ht="15.75" customHeight="1">
-      <x:c r="F40" s="10"/>
-      <x:c r="I40" s="10"/>
+      <x:c r="F40" s="9"/>
+      <x:c r="I40" s="9"/>
     </x:row>
     <x:row r="41" ht="15.75" customHeight="1">
-      <x:c r="F41" s="10"/>
-      <x:c r="I41" s="10"/>
+      <x:c r="F41" s="9"/>
+      <x:c r="I41" s="9"/>
     </x:row>
     <x:row r="42" ht="15.75" customHeight="1">
-      <x:c r="F42" s="10"/>
-      <x:c r="I42" s="10"/>
+      <x:c r="F42" s="9"/>
+      <x:c r="I42" s="9"/>
     </x:row>
     <x:row r="43" ht="15.75" customHeight="1">
-      <x:c r="F43" s="10"/>
-      <x:c r="I43" s="10"/>
+      <x:c r="F43" s="9"/>
+      <x:c r="I43" s="9"/>
     </x:row>
     <x:row r="44" ht="15.75" customHeight="1">
-      <x:c r="F44" s="10"/>
-      <x:c r="I44" s="10"/>
+      <x:c r="F44" s="9"/>
+      <x:c r="I44" s="9"/>
     </x:row>
     <x:row r="45" ht="15.75" customHeight="1">
-      <x:c r="F45" s="10"/>
-      <x:c r="I45" s="10"/>
+      <x:c r="F45" s="9"/>
+      <x:c r="I45" s="9"/>
     </x:row>
     <x:row r="46" ht="15.75" customHeight="1">
-      <x:c r="F46" s="10"/>
-      <x:c r="I46" s="10"/>
+      <x:c r="F46" s="9"/>
+      <x:c r="I46" s="9"/>
     </x:row>
     <x:row r="47" ht="15.75" customHeight="1">
-      <x:c r="F47" s="10"/>
-      <x:c r="I47" s="10"/>
+      <x:c r="F47" s="9"/>
+      <x:c r="I47" s="9"/>
     </x:row>
     <x:row r="48" ht="15.75" customHeight="1">
-      <x:c r="F48" s="10"/>
-      <x:c r="I48" s="10"/>
+      <x:c r="F48" s="9"/>
+      <x:c r="I48" s="9"/>
     </x:row>
     <x:row r="49" ht="15.75" customHeight="1">
-      <x:c r="F49" s="10"/>
-      <x:c r="I49" s="10"/>
+      <x:c r="F49" s="9"/>
+      <x:c r="I49" s="9"/>
     </x:row>
     <x:row r="50" ht="15.75" customHeight="1">
-      <x:c r="F50" s="10"/>
-      <x:c r="I50" s="10"/>
+      <x:c r="F50" s="9"/>
+      <x:c r="I50" s="9"/>
     </x:row>
     <x:row r="51" ht="15.75" customHeight="1">
-      <x:c r="F51" s="10"/>
-      <x:c r="I51" s="10"/>
+      <x:c r="F51" s="9"/>
+      <x:c r="I51" s="9"/>
     </x:row>
     <x:row r="52" ht="15.75" customHeight="1">
-      <x:c r="F52" s="10"/>
-      <x:c r="I52" s="10"/>
+      <x:c r="F52" s="9"/>
+      <x:c r="I52" s="9"/>
     </x:row>
     <x:row r="53" ht="15.75" customHeight="1">
-      <x:c r="F53" s="10"/>
-      <x:c r="I53" s="10"/>
+      <x:c r="F53" s="9"/>
+      <x:c r="I53" s="9"/>
     </x:row>
     <x:row r="54" ht="15.75" customHeight="1">
-      <x:c r="F54" s="10"/>
-      <x:c r="I54" s="10"/>
+      <x:c r="F54" s="9"/>
+      <x:c r="I54" s="9"/>
     </x:row>
     <x:row r="55" ht="15.75" customHeight="1">
-      <x:c r="F55" s="10"/>
-      <x:c r="I55" s="10"/>
+      <x:c r="F55" s="9"/>
+      <x:c r="I55" s="9"/>
     </x:row>
     <x:row r="56" ht="15.75" customHeight="1">
-      <x:c r="F56" s="10"/>
-      <x:c r="I56" s="10"/>
+      <x:c r="F56" s="9"/>
+      <x:c r="I56" s="9"/>
     </x:row>
     <x:row r="57" ht="15.75" customHeight="1">
-      <x:c r="F57" s="10"/>
-      <x:c r="I57" s="10"/>
+      <x:c r="F57" s="9"/>
+      <x:c r="I57" s="9"/>
     </x:row>
     <x:row r="58" ht="15.75" customHeight="1">
-      <x:c r="F58" s="10"/>
-      <x:c r="I58" s="10"/>
+      <x:c r="F58" s="9"/>
+      <x:c r="I58" s="9"/>
     </x:row>
     <x:row r="59" ht="15.75" customHeight="1">
-      <x:c r="F59" s="10"/>
-      <x:c r="I59" s="10"/>
+      <x:c r="F59" s="9"/>
+      <x:c r="I59" s="9"/>
     </x:row>
     <x:row r="60" ht="15.75" customHeight="1">
-      <x:c r="F60" s="10"/>
-      <x:c r="I60" s="10"/>
+      <x:c r="F60" s="9"/>
+      <x:c r="I60" s="9"/>
     </x:row>
     <x:row r="61" ht="15.75" customHeight="1">
-      <x:c r="F61" s="10"/>
-      <x:c r="I61" s="10"/>
+      <x:c r="F61" s="9"/>
+      <x:c r="I61" s="9"/>
     </x:row>
     <x:row r="62" ht="15.75" customHeight="1">
-      <x:c r="F62" s="10"/>
-      <x:c r="I62" s="10"/>
+      <x:c r="F62" s="9"/>
+      <x:c r="I62" s="9"/>
     </x:row>
     <x:row r="63" ht="15.75" customHeight="1">
-      <x:c r="F63" s="10"/>
-      <x:c r="I63" s="10"/>
+      <x:c r="F63" s="9"/>
+      <x:c r="I63" s="9"/>
     </x:row>
     <x:row r="64" ht="15.75" customHeight="1">
-      <x:c r="F64" s="10"/>
-      <x:c r="I64" s="10"/>
+      <x:c r="F64" s="9"/>
+      <x:c r="I64" s="9"/>
     </x:row>
     <x:row r="65" ht="15.75" customHeight="1">
-      <x:c r="F65" s="10"/>
-      <x:c r="I65" s="10"/>
+      <x:c r="F65" s="9"/>
+      <x:c r="I65" s="9"/>
     </x:row>
     <x:row r="66" ht="15.75" customHeight="1">
-      <x:c r="F66" s="10"/>
-      <x:c r="I66" s="10"/>
+      <x:c r="F66" s="9"/>
+      <x:c r="I66" s="9"/>
     </x:row>
     <x:row r="67" ht="15.75" customHeight="1">
-      <x:c r="F67" s="10"/>
-      <x:c r="I67" s="10"/>
+      <x:c r="F67" s="9"/>
+      <x:c r="I67" s="9"/>
     </x:row>
     <x:row r="68" ht="15.75" customHeight="1">
-      <x:c r="F68" s="10"/>
-      <x:c r="I68" s="10"/>
+      <x:c r="F68" s="9"/>
+      <x:c r="I68" s="9"/>
     </x:row>
     <x:row r="69" ht="15.75" customHeight="1">
-      <x:c r="F69" s="10"/>
-      <x:c r="I69" s="10"/>
+      <x:c r="F69" s="9"/>
+      <x:c r="I69" s="9"/>
     </x:row>
     <x:row r="70" ht="15.75" customHeight="1">
-      <x:c r="F70" s="10"/>
-      <x:c r="I70" s="10"/>
+      <x:c r="F70" s="9"/>
+      <x:c r="I70" s="9"/>
     </x:row>
     <x:row r="71" ht="15.75" customHeight="1">
-      <x:c r="F71" s="10"/>
-      <x:c r="I71" s="10"/>
+      <x:c r="F71" s="9"/>
+      <x:c r="I71" s="9"/>
     </x:row>
     <x:row r="72" ht="15.75" customHeight="1">
-      <x:c r="F72" s="10"/>
-      <x:c r="I72" s="10"/>
+      <x:c r="F72" s="9"/>
+      <x:c r="I72" s="9"/>
     </x:row>
     <x:row r="73" ht="15.75" customHeight="1">
-      <x:c r="F73" s="10"/>
-      <x:c r="I73" s="10"/>
+      <x:c r="F73" s="9"/>
+      <x:c r="I73" s="9"/>
     </x:row>
     <x:row r="74" ht="15.75" customHeight="1">
-      <x:c r="F74" s="10"/>
-      <x:c r="I74" s="10"/>
+      <x:c r="F74" s="9"/>
+      <x:c r="I74" s="9"/>
     </x:row>
     <x:row r="75" ht="15.75" customHeight="1">
-      <x:c r="F75" s="10"/>
-      <x:c r="I75" s="10"/>
+      <x:c r="F75" s="9"/>
+      <x:c r="I75" s="9"/>
     </x:row>
     <x:row r="76" ht="15.75" customHeight="1">
-      <x:c r="F76" s="10"/>
-      <x:c r="I76" s="10"/>
+      <x:c r="F76" s="9"/>
+      <x:c r="I76" s="9"/>
     </x:row>
     <x:row r="77" ht="15.75" customHeight="1">
-      <x:c r="F77" s="10"/>
-      <x:c r="I77" s="10"/>
+      <x:c r="F77" s="9"/>
+      <x:c r="I77" s="9"/>
     </x:row>
     <x:row r="78" ht="15.75" customHeight="1">
-      <x:c r="F78" s="10"/>
-      <x:c r="I78" s="10"/>
+      <x:c r="F78" s="9"/>
+      <x:c r="I78" s="9"/>
     </x:row>
     <x:row r="79" ht="15.75" customHeight="1">
-      <x:c r="F79" s="10"/>
-      <x:c r="I79" s="10"/>
+      <x:c r="F79" s="9"/>
+      <x:c r="I79" s="9"/>
     </x:row>
     <x:row r="80" ht="15.75" customHeight="1">
-      <x:c r="F80" s="10"/>
-      <x:c r="I80" s="10"/>
+      <x:c r="F80" s="9"/>
+      <x:c r="I80" s="9"/>
     </x:row>
     <x:row r="81" ht="15.75" customHeight="1">
-      <x:c r="F81" s="10"/>
-      <x:c r="I81" s="10"/>
+      <x:c r="F81" s="9"/>
+      <x:c r="I81" s="9"/>
     </x:row>
     <x:row r="82" ht="15.75" customHeight="1">
-      <x:c r="F82" s="10"/>
-      <x:c r="I82" s="10"/>
+      <x:c r="F82" s="9"/>
+      <x:c r="I82" s="9"/>
     </x:row>
     <x:row r="83" ht="15.75" customHeight="1">
-      <x:c r="F83" s="10"/>
-      <x:c r="I83" s="10"/>
+      <x:c r="F83" s="9"/>
+      <x:c r="I83" s="9"/>
     </x:row>
     <x:row r="84" ht="15.75" customHeight="1">
-      <x:c r="F84" s="10"/>
-      <x:c r="I84" s="10"/>
+      <x:c r="F84" s="9"/>
+      <x:c r="I84" s="9"/>
     </x:row>
     <x:row r="85" ht="15.75" customHeight="1">
-      <x:c r="F85" s="10"/>
-      <x:c r="I85" s="10"/>
+      <x:c r="F85" s="9"/>
+      <x:c r="I85" s="9"/>
     </x:row>
     <x:row r="86" ht="15.75" customHeight="1">
-      <x:c r="F86" s="10"/>
-      <x:c r="I86" s="10"/>
+      <x:c r="F86" s="9"/>
+      <x:c r="I86" s="9"/>
     </x:row>
     <x:row r="87" ht="15.75" customHeight="1">
-      <x:c r="F87" s="10"/>
-      <x:c r="I87" s="10"/>
+      <x:c r="F87" s="9"/>
+      <x:c r="I87" s="9"/>
     </x:row>
     <x:row r="88" ht="15.75" customHeight="1">
-      <x:c r="F88" s="10"/>
-      <x:c r="I88" s="10"/>
+      <x:c r="F88" s="9"/>
+      <x:c r="I88" s="9"/>
     </x:row>
     <x:row r="89" ht="15.75" customHeight="1">
-      <x:c r="F89" s="10"/>
-      <x:c r="I89" s="10"/>
+      <x:c r="F89" s="9"/>
+      <x:c r="I89" s="9"/>
     </x:row>
     <x:row r="90" ht="15.75" customHeight="1">
-      <x:c r="F90" s="10"/>
-      <x:c r="I90" s="10"/>
+      <x:c r="F90" s="9"/>
+      <x:c r="I90" s="9"/>
     </x:row>
     <x:row r="91" ht="15.75" customHeight="1">
-      <x:c r="F91" s="10"/>
-      <x:c r="I91" s="10"/>
+      <x:c r="F91" s="9"/>
+      <x:c r="I91" s="9"/>
     </x:row>
     <x:row r="92" ht="15.75" customHeight="1">
-      <x:c r="F92" s="10"/>
-      <x:c r="I92" s="10"/>
+      <x:c r="F92" s="9"/>
+      <x:c r="I92" s="9"/>
     </x:row>
     <x:row r="93" ht="15.75" customHeight="1">
-      <x:c r="F93" s="10"/>
-      <x:c r="I93" s="10"/>
+      <x:c r="F93" s="9"/>
+      <x:c r="I93" s="9"/>
     </x:row>
     <x:row r="94" ht="15.75" customHeight="1">
-      <x:c r="F94" s="10"/>
-      <x:c r="I94" s="10"/>
+      <x:c r="F94" s="9"/>
+      <x:c r="I94" s="9"/>
     </x:row>
     <x:row r="95" ht="15.75" customHeight="1">
-      <x:c r="F95" s="10"/>
-      <x:c r="I95" s="10"/>
+      <x:c r="F95" s="9"/>
+      <x:c r="I95" s="9"/>
     </x:row>
     <x:row r="96" ht="15.75" customHeight="1">
-      <x:c r="F96" s="10"/>
-      <x:c r="I96" s="10"/>
+      <x:c r="F96" s="9"/>
+      <x:c r="I96" s="9"/>
     </x:row>
     <x:row r="97" ht="15.75" customHeight="1">
-      <x:c r="F97" s="10"/>
-      <x:c r="I97" s="10"/>
+      <x:c r="F97" s="9"/>
+      <x:c r="I97" s="9"/>
     </x:row>
     <x:row r="98" ht="15.75" customHeight="1">
-      <x:c r="F98" s="10"/>
-      <x:c r="I98" s="10"/>
+      <x:c r="F98" s="9"/>
+      <x:c r="I98" s="9"/>
     </x:row>
     <x:row r="99" ht="15.75" customHeight="1">
-      <x:c r="F99" s="10"/>
-      <x:c r="I99" s="10"/>
+      <x:c r="F99" s="9"/>
+      <x:c r="I99" s="9"/>
     </x:row>
     <x:row r="100" ht="15.75" customHeight="1">
-      <x:c r="F100" s="10"/>
-      <x:c r="I100" s="10"/>
+      <x:c r="F100" s="9"/>
+      <x:c r="I100" s="9"/>
     </x:row>
     <x:row r="101" ht="15.75" customHeight="1">
-      <x:c r="F101" s="10"/>
-      <x:c r="I101" s="10"/>
+      <x:c r="F101" s="9"/>
+      <x:c r="I101" s="9"/>
     </x:row>
     <x:row r="102" ht="15.75" customHeight="1">
-      <x:c r="F102" s="10"/>
-      <x:c r="I102" s="10"/>
+      <x:c r="F102" s="9"/>
+      <x:c r="I102" s="9"/>
     </x:row>
     <x:row r="103" ht="15.75" customHeight="1">
-      <x:c r="F103" s="10"/>
-      <x:c r="I103" s="10"/>
+      <x:c r="F103" s="9"/>
+      <x:c r="I103" s="9"/>
     </x:row>
     <x:row r="104" ht="15.75" customHeight="1">
-      <x:c r="F104" s="10"/>
-      <x:c r="I104" s="10"/>
+      <x:c r="F104" s="9"/>
+      <x:c r="I104" s="9"/>
     </x:row>
     <x:row r="105" ht="15.75" customHeight="1">
-      <x:c r="F105" s="10"/>
-      <x:c r="I105" s="10"/>
+      <x:c r="F105" s="9"/>
+      <x:c r="I105" s="9"/>
     </x:row>
     <x:row r="106" ht="15.75" customHeight="1">
-      <x:c r="F106" s="10"/>
-      <x:c r="I106" s="10"/>
+      <x:c r="F106" s="9"/>
+      <x:c r="I106" s="9"/>
     </x:row>
     <x:row r="107" ht="15.75" customHeight="1">
-      <x:c r="F107" s="10"/>
-      <x:c r="I107" s="10"/>
+      <x:c r="F107" s="9"/>
+      <x:c r="I107" s="9"/>
     </x:row>
     <x:row r="108" ht="15.75" customHeight="1">
-      <x:c r="F108" s="10"/>
-      <x:c r="I108" s="10"/>
+      <x:c r="F108" s="9"/>
+      <x:c r="I108" s="9"/>
     </x:row>
     <x:row r="109" ht="15.75" customHeight="1">
-      <x:c r="F109" s="10"/>
-      <x:c r="I109" s="10"/>
+      <x:c r="F109" s="9"/>
+      <x:c r="I109" s="9"/>
     </x:row>
     <x:row r="110" ht="15.75" customHeight="1">
-      <x:c r="F110" s="10"/>
-      <x:c r="I110" s="10"/>
+      <x:c r="F110" s="9"/>
+      <x:c r="I110" s="9"/>
     </x:row>
     <x:row r="111" ht="15.75" customHeight="1">
-      <x:c r="F111" s="10"/>
-      <x:c r="I111" s="10"/>
+      <x:c r="F111" s="9"/>
+      <x:c r="I111" s="9"/>
     </x:row>
     <x:row r="112" ht="15.75" customHeight="1">
-      <x:c r="F112" s="10"/>
-      <x:c r="I112" s="10"/>
+      <x:c r="F112" s="9"/>
+      <x:c r="I112" s="9"/>
     </x:row>
     <x:row r="113" ht="15.75" customHeight="1">
-      <x:c r="F113" s="10"/>
-      <x:c r="I113" s="10"/>
+      <x:c r="F113" s="9"/>
+      <x:c r="I113" s="9"/>
     </x:row>
     <x:row r="114" ht="15.75" customHeight="1">
-      <x:c r="F114" s="10"/>
-      <x:c r="I114" s="10"/>
+      <x:c r="F114" s="9"/>
+      <x:c r="I114" s="9"/>
     </x:row>
     <x:row r="115" ht="15.75" customHeight="1">
-      <x:c r="F115" s="10"/>
-      <x:c r="I115" s="10"/>
+      <x:c r="F115" s="9"/>
+      <x:c r="I115" s="9"/>
     </x:row>
     <x:row r="116" ht="15.75" customHeight="1">
-      <x:c r="F116" s="10"/>
-      <x:c r="I116" s="10"/>
+      <x:c r="F116" s="9"/>
+      <x:c r="I116" s="9"/>
     </x:row>
     <x:row r="117" ht="15.75" customHeight="1">
-      <x:c r="F117" s="10"/>
-      <x:c r="I117" s="10"/>
+      <x:c r="F117" s="9"/>
+      <x:c r="I117" s="9"/>
     </x:row>
     <x:row r="118" ht="15.75" customHeight="1">
-      <x:c r="F118" s="10"/>
-      <x:c r="I118" s="10"/>
+      <x:c r="F118" s="9"/>
+      <x:c r="I118" s="9"/>
     </x:row>
     <x:row r="119" ht="15.75" customHeight="1">
-      <x:c r="F119" s="10"/>
-      <x:c r="I119" s="10"/>
+      <x:c r="F119" s="9"/>
+      <x:c r="I119" s="9"/>
     </x:row>
     <x:row r="120" ht="15.75" customHeight="1">
-      <x:c r="F120" s="10"/>
-      <x:c r="I120" s="10"/>
+      <x:c r="F120" s="9"/>
+      <x:c r="I120" s="9"/>
     </x:row>
     <x:row r="121" ht="15.75" customHeight="1">
-      <x:c r="F121" s="10"/>
-      <x:c r="I121" s="10"/>
+      <x:c r="F121" s="9"/>
+      <x:c r="I121" s="9"/>
     </x:row>
     <x:row r="122" ht="15.75" customHeight="1">
-      <x:c r="F122" s="10"/>
-      <x:c r="I122" s="10"/>
+      <x:c r="F122" s="9"/>
+      <x:c r="I122" s="9"/>
     </x:row>
     <x:row r="123" ht="15.75" customHeight="1">
-      <x:c r="F123" s="10"/>
-      <x:c r="I123" s="10"/>
+      <x:c r="F123" s="9"/>
+      <x:c r="I123" s="9"/>
     </x:row>
     <x:row r="124" ht="15.75" customHeight="1">
-      <x:c r="F124" s="10"/>
-      <x:c r="I124" s="10"/>
+      <x:c r="F124" s="9"/>
+      <x:c r="I124" s="9"/>
     </x:row>
     <x:row r="125" ht="15.75" customHeight="1">
-      <x:c r="F125" s="10"/>
-      <x:c r="I125" s="10"/>
+      <x:c r="F125" s="9"/>
+      <x:c r="I125" s="9"/>
     </x:row>
     <x:row r="126" ht="15.75" customHeight="1">
-      <x:c r="F126" s="10"/>
-      <x:c r="I126" s="10"/>
+      <x:c r="F126" s="9"/>
+      <x:c r="I126" s="9"/>
     </x:row>
     <x:row r="127" ht="15.75" customHeight="1">
-      <x:c r="F127" s="10"/>
-      <x:c r="I127" s="10"/>
+      <x:c r="F127" s="9"/>
+      <x:c r="I127" s="9"/>
     </x:row>
     <x:row r="128" ht="15.75" customHeight="1">
-      <x:c r="F128" s="10"/>
-      <x:c r="I128" s="10"/>
+      <x:c r="F128" s="9"/>
+      <x:c r="I128" s="9"/>
     </x:row>
     <x:row r="129" ht="15.75" customHeight="1">
-      <x:c r="F129" s="10"/>
-      <x:c r="I129" s="10"/>
+      <x:c r="F129" s="9"/>
+      <x:c r="I129" s="9"/>
     </x:row>
     <x:row r="130" ht="15.75" customHeight="1">
-      <x:c r="F130" s="10"/>
-      <x:c r="I130" s="10"/>
+      <x:c r="F130" s="9"/>
+      <x:c r="I130" s="9"/>
     </x:row>
     <x:row r="131" ht="15.75" customHeight="1">
-      <x:c r="F131" s="10"/>
-      <x:c r="I131" s="10"/>
+      <x:c r="F131" s="9"/>
+      <x:c r="I131" s="9"/>
     </x:row>
     <x:row r="132" ht="15.75" customHeight="1">
-      <x:c r="F132" s="10"/>
-      <x:c r="I132" s="10"/>
+      <x:c r="F132" s="9"/>
+      <x:c r="I132" s="9"/>
     </x:row>
     <x:row r="133" ht="15.75" customHeight="1">
-      <x:c r="F133" s="10"/>
-      <x:c r="I133" s="10"/>
+      <x:c r="F133" s="9"/>
+      <x:c r="I133" s="9"/>
     </x:row>
     <x:row r="134" ht="15.75" customHeight="1">
-      <x:c r="F134" s="10"/>
-      <x:c r="I134" s="10"/>
+      <x:c r="F134" s="9"/>
+      <x:c r="I134" s="9"/>
     </x:row>
     <x:row r="135" ht="15.75" customHeight="1">
-      <x:c r="F135" s="10"/>
-      <x:c r="I135" s="10"/>
+      <x:c r="F135" s="9"/>
+      <x:c r="I135" s="9"/>
     </x:row>
     <x:row r="136" ht="15.75" customHeight="1">
-      <x:c r="F136" s="10"/>
-      <x:c r="I136" s="10"/>
+      <x:c r="F136" s="9"/>
+      <x:c r="I136" s="9"/>
     </x:row>
     <x:row r="137" ht="15.75" customHeight="1">
-      <x:c r="F137" s="10"/>
-      <x:c r="I137" s="10"/>
+      <x:c r="F137" s="9"/>
+      <x:c r="I137" s="9"/>
     </x:row>
     <x:row r="138" ht="15.75" customHeight="1">
-      <x:c r="F138" s="10"/>
-      <x:c r="I138" s="10"/>
+      <x:c r="F138" s="9"/>
+      <x:c r="I138" s="9"/>
     </x:row>
     <x:row r="139" ht="15.75" customHeight="1">
-      <x:c r="F139" s="10"/>
-      <x:c r="I139" s="10"/>
+      <x:c r="F139" s="9"/>
+      <x:c r="I139" s="9"/>
     </x:row>
     <x:row r="140" ht="15.75" customHeight="1">
-      <x:c r="F140" s="10"/>
-      <x:c r="I140" s="10"/>
+      <x:c r="F140" s="9"/>
+      <x:c r="I140" s="9"/>
     </x:row>
     <x:row r="141" ht="15.75" customHeight="1">
-      <x:c r="F141" s="10"/>
-      <x:c r="I141" s="10"/>
+      <x:c r="F141" s="9"/>
+      <x:c r="I141" s="9"/>
     </x:row>
     <x:row r="142" ht="15.75" customHeight="1">
-      <x:c r="F142" s="10"/>
-      <x:c r="I142" s="10"/>
+      <x:c r="F142" s="9"/>
+      <x:c r="I142" s="9"/>
     </x:row>
     <x:row r="143" ht="15.75" customHeight="1">
-      <x:c r="F143" s="10"/>
-      <x:c r="I143" s="10"/>
+      <x:c r="F143" s="9"/>
+      <x:c r="I143" s="9"/>
     </x:row>
     <x:row r="144" ht="15.75" customHeight="1">
-      <x:c r="F144" s="10"/>
-      <x:c r="I144" s="10"/>
+      <x:c r="F144" s="9"/>
+      <x:c r="I144" s="9"/>
     </x:row>
     <x:row r="145" ht="15.75" customHeight="1">
-      <x:c r="F145" s="10"/>
-      <x:c r="I145" s="10"/>
+      <x:c r="F145" s="9"/>
+      <x:c r="I145" s="9"/>
     </x:row>
     <x:row r="146" ht="15.75" customHeight="1">
-      <x:c r="F146" s="10"/>
-      <x:c r="I146" s="10"/>
+      <x:c r="F146" s="9"/>
+      <x:c r="I146" s="9"/>
     </x:row>
     <x:row r="147" ht="15.75" customHeight="1">
-      <x:c r="F147" s="10"/>
-      <x:c r="I147" s="10"/>
+      <x:c r="F147" s="9"/>
+      <x:c r="I147" s="9"/>
     </x:row>
     <x:row r="148" ht="15.75" customHeight="1">
-      <x:c r="F148" s="10"/>
-      <x:c r="I148" s="10"/>
+      <x:c r="F148" s="9"/>
+      <x:c r="I148" s="9"/>
     </x:row>
     <x:row r="149" ht="15.75" customHeight="1">
-      <x:c r="F149" s="10"/>
-      <x:c r="I149" s="10"/>
+      <x:c r="F149" s="9"/>
+      <x:c r="I149" s="9"/>
     </x:row>
     <x:row r="150" ht="15.75" customHeight="1">
-      <x:c r="F150" s="10"/>
-      <x:c r="I150" s="10"/>
+      <x:c r="F150" s="9"/>
+      <x:c r="I150" s="9"/>
     </x:row>
     <x:row r="151" ht="15.75" customHeight="1">
-      <x:c r="F151" s="10"/>
-      <x:c r="I151" s="10"/>
+      <x:c r="F151" s="9"/>
+      <x:c r="I151" s="9"/>
     </x:row>
     <x:row r="152" ht="15.75" customHeight="1">
-      <x:c r="F152" s="10"/>
-      <x:c r="I152" s="10"/>
+      <x:c r="F152" s="9"/>
+      <x:c r="I152" s="9"/>
     </x:row>
     <x:row r="153" ht="15.75" customHeight="1">
-      <x:c r="F153" s="10"/>
-      <x:c r="I153" s="10"/>
+      <x:c r="F153" s="9"/>
+      <x:c r="I153" s="9"/>
     </x:row>
     <x:row r="154" ht="15.75" customHeight="1">
-      <x:c r="F154" s="10"/>
-      <x:c r="I154" s="10"/>
+      <x:c r="F154" s="9"/>
+      <x:c r="I154" s="9"/>
     </x:row>
     <x:row r="155" ht="15.75" customHeight="1">
-      <x:c r="F155" s="10"/>
-      <x:c r="I155" s="10"/>
+      <x:c r="F155" s="9"/>
+      <x:c r="I155" s="9"/>
     </x:row>
     <x:row r="156" ht="15.75" customHeight="1">
-      <x:c r="F156" s="10"/>
-      <x:c r="I156" s="10"/>
+      <x:c r="F156" s="9"/>
+      <x:c r="I156" s="9"/>
     </x:row>
     <x:row r="157" ht="15.75" customHeight="1">
-      <x:c r="F157" s="10"/>
-      <x:c r="I157" s="10"/>
+      <x:c r="F157" s="9"/>
+      <x:c r="I157" s="9"/>
     </x:row>
     <x:row r="158" ht="15.75" customHeight="1">
-      <x:c r="F158" s="10"/>
-      <x:c r="I158" s="10"/>
+      <x:c r="F158" s="9"/>
+      <x:c r="I158" s="9"/>
     </x:row>
     <x:row r="159" ht="15.75" customHeight="1">
-      <x:c r="F159" s="10"/>
-      <x:c r="I159" s="10"/>
+      <x:c r="F159" s="9"/>
+      <x:c r="I159" s="9"/>
     </x:row>
     <x:row r="160" ht="15.75" customHeight="1">
-      <x:c r="F160" s="10"/>
-      <x:c r="I160" s="10"/>
+      <x:c r="F160" s="9"/>
+      <x:c r="I160" s="9"/>
     </x:row>
     <x:row r="161" ht="15.75" customHeight="1">
-      <x:c r="F161" s="10"/>
-      <x:c r="I161" s="10"/>
+      <x:c r="F161" s="9"/>
+      <x:c r="I161" s="9"/>
     </x:row>
     <x:row r="162" ht="15.75" customHeight="1">
-      <x:c r="F162" s="10"/>
-      <x:c r="I162" s="10"/>
+      <x:c r="F162" s="9"/>
+      <x:c r="I162" s="9"/>
     </x:row>
     <x:row r="163" ht="15.75" customHeight="1">
-      <x:c r="F163" s="10"/>
-      <x:c r="I163" s="10"/>
+      <x:c r="F163" s="9"/>
+      <x:c r="I163" s="9"/>
     </x:row>
     <x:row r="164" ht="15.75" customHeight="1">
-      <x:c r="F164" s="10"/>
-      <x:c r="I164" s="10"/>
+      <x:c r="F164" s="9"/>
+      <x:c r="I164" s="9"/>
     </x:row>
     <x:row r="165" ht="15.75" customHeight="1">
-      <x:c r="F165" s="10"/>
-      <x:c r="I165" s="10"/>
+      <x:c r="F165" s="9"/>
+      <x:c r="I165" s="9"/>
     </x:row>
     <x:row r="166" ht="15.75" customHeight="1">
-      <x:c r="F166" s="10"/>
-      <x:c r="I166" s="10"/>
+      <x:c r="F166" s="9"/>
+      <x:c r="I166" s="9"/>
     </x:row>
     <x:row r="167" ht="15.75" customHeight="1">
-      <x:c r="F167" s="10"/>
-      <x:c r="I167" s="10"/>
+      <x:c r="F167" s="9"/>
+      <x:c r="I167" s="9"/>
     </x:row>
     <x:row r="168" ht="15.75" customHeight="1">
-      <x:c r="F168" s="10"/>
-      <x:c r="I168" s="10"/>
+      <x:c r="F168" s="9"/>
+      <x:c r="I168" s="9"/>
     </x:row>
     <x:row r="169" ht="15.75" customHeight="1">
-      <x:c r="F169" s="10"/>
-      <x:c r="I169" s="10"/>
+      <x:c r="F169" s="9"/>
+      <x:c r="I169" s="9"/>
     </x:row>
     <x:row r="170" ht="15.75" customHeight="1">
-      <x:c r="F170" s="10"/>
-      <x:c r="I170" s="10"/>
+      <x:c r="F170" s="9"/>
+      <x:c r="I170" s="9"/>
     </x:row>
     <x:row r="171" ht="15.75" customHeight="1">
-      <x:c r="F171" s="10"/>
-      <x:c r="I171" s="10"/>
+      <x:c r="F171" s="9"/>
+      <x:c r="I171" s="9"/>
     </x:row>
     <x:row r="172" ht="15.75" customHeight="1">
-      <x:c r="F172" s="10"/>
-      <x:c r="I172" s="10"/>
+      <x:c r="F172" s="9"/>
+      <x:c r="I172" s="9"/>
     </x:row>
     <x:row r="173" ht="15.75" customHeight="1">
-      <x:c r="F173" s="10"/>
-      <x:c r="I173" s="10"/>
+      <x:c r="F173" s="9"/>
+      <x:c r="I173" s="9"/>
     </x:row>
     <x:row r="174" ht="15.75" customHeight="1">
-      <x:c r="F174" s="10"/>
-      <x:c r="I174" s="10"/>
+      <x:c r="F174" s="9"/>
+      <x:c r="I174" s="9"/>
     </x:row>
     <x:row r="175" ht="15.75" customHeight="1">
-      <x:c r="F175" s="10"/>
-      <x:c r="I175" s="10"/>
+      <x:c r="F175" s="9"/>
+      <x:c r="I175" s="9"/>
     </x:row>
     <x:row r="176" ht="15.75" customHeight="1">
-      <x:c r="F176" s="10"/>
-      <x:c r="I176" s="10"/>
+      <x:c r="F176" s="9"/>
+      <x:c r="I176" s="9"/>
     </x:row>
     <x:row r="177" ht="15.75" customHeight="1">
-      <x:c r="F177" s="10"/>
-      <x:c r="I177" s="10"/>
+      <x:c r="F177" s="9"/>
+      <x:c r="I177" s="9"/>
     </x:row>
     <x:row r="178" ht="15.75" customHeight="1">
-      <x:c r="F178" s="10"/>
-      <x:c r="I178" s="10"/>
+      <x:c r="F178" s="9"/>
+      <x:c r="I178" s="9"/>
     </x:row>
     <x:row r="179" ht="15.75" customHeight="1">
-      <x:c r="F179" s="10"/>
-      <x:c r="I179" s="10"/>
+      <x:c r="F179" s="9"/>
+      <x:c r="I179" s="9"/>
     </x:row>
     <x:row r="180" ht="15.75" customHeight="1">
-      <x:c r="F180" s="10"/>
-      <x:c r="I180" s="10"/>
+      <x:c r="F180" s="9"/>
+      <x:c r="I180" s="9"/>
     </x:row>
     <x:row r="181" ht="15.75" customHeight="1">
-      <x:c r="F181" s="10"/>
-      <x:c r="I181" s="10"/>
+      <x:c r="F181" s="9"/>
+      <x:c r="I181" s="9"/>
     </x:row>
     <x:row r="182" ht="15.75" customHeight="1">
-      <x:c r="F182" s="10"/>
-      <x:c r="I182" s="10"/>
+      <x:c r="F182" s="9"/>
+      <x:c r="I182" s="9"/>
     </x:row>
     <x:row r="183" ht="15.75" customHeight="1">
-      <x:c r="F183" s="10"/>
-      <x:c r="I183" s="10"/>
+      <x:c r="F183" s="9"/>
+      <x:c r="I183" s="9"/>
     </x:row>
     <x:row r="184" ht="15.75" customHeight="1">
-      <x:c r="F184" s="10"/>
-      <x:c r="I184" s="10"/>
+      <x:c r="F184" s="9"/>
+      <x:c r="I184" s="9"/>
     </x:row>
     <x:row r="185" ht="15.75" customHeight="1">
-      <x:c r="F185" s="10"/>
-      <x:c r="I185" s="10"/>
+      <x:c r="F185" s="9"/>
+      <x:c r="I185" s="9"/>
     </x:row>
     <x:row r="186" ht="15.75" customHeight="1">
-      <x:c r="F186" s="10"/>
-      <x:c r="I186" s="10"/>
+      <x:c r="F186" s="9"/>
+      <x:c r="I186" s="9"/>
     </x:row>
     <x:row r="187" ht="15.75" customHeight="1">
-      <x:c r="F187" s="10"/>
-      <x:c r="I187" s="10"/>
+      <x:c r="F187" s="9"/>
+      <x:c r="I187" s="9"/>
     </x:row>
     <x:row r="188" ht="15.75" customHeight="1">
-      <x:c r="F188" s="10"/>
-      <x:c r="I188" s="10"/>
+      <x:c r="F188" s="9"/>
+      <x:c r="I188" s="9"/>
     </x:row>
     <x:row r="189" ht="15.75" customHeight="1">
-      <x:c r="F189" s="10"/>
-      <x:c r="I189" s="10"/>
+      <x:c r="F189" s="9"/>
+      <x:c r="I189" s="9"/>
     </x:row>
     <x:row r="190" ht="15.75" customHeight="1">
-      <x:c r="F190" s="10"/>
-      <x:c r="I190" s="10"/>
+      <x:c r="F190" s="9"/>
+      <x:c r="I190" s="9"/>
     </x:row>
     <x:row r="191" ht="15.75" customHeight="1">
-      <x:c r="F191" s="10"/>
-      <x:c r="I191" s="10"/>
+      <x:c r="F191" s="9"/>
+      <x:c r="I191" s="9"/>
     </x:row>
     <x:row r="192" ht="15.75" customHeight="1">
-      <x:c r="F192" s="10"/>
-      <x:c r="I192" s="10"/>
+      <x:c r="F192" s="9"/>
+      <x:c r="I192" s="9"/>
     </x:row>
     <x:row r="193" ht="15.75" customHeight="1">
-      <x:c r="F193" s="10"/>
-      <x:c r="I193" s="10"/>
+      <x:c r="F193" s="9"/>
+      <x:c r="I193" s="9"/>
     </x:row>
     <x:row r="194" ht="15.75" customHeight="1">
-      <x:c r="F194" s="10"/>
-      <x:c r="I194" s="10"/>
+      <x:c r="F194" s="9"/>
+      <x:c r="I194" s="9"/>
     </x:row>
     <x:row r="195" ht="15.75" customHeight="1">
-      <x:c r="F195" s="10"/>
-      <x:c r="I195" s="10"/>
+      <x:c r="F195" s="9"/>
+      <x:c r="I195" s="9"/>
     </x:row>
     <x:row r="196" ht="15.75" customHeight="1">
-      <x:c r="F196" s="10"/>
-      <x:c r="I196" s="10"/>
+      <x:c r="F196" s="9"/>
+      <x:c r="I196" s="9"/>
     </x:row>
     <x:row r="197" ht="15.75" customHeight="1">
-      <x:c r="F197" s="10"/>
-      <x:c r="I197" s="10"/>
+      <x:c r="F197" s="9"/>
+      <x:c r="I197" s="9"/>
     </x:row>
     <x:row r="198" ht="15.75" customHeight="1">
-      <x:c r="F198" s="10"/>
-      <x:c r="I198" s="10"/>
+      <x:c r="F198" s="9"/>
+      <x:c r="I198" s="9"/>
     </x:row>
     <x:row r="199" ht="15.75" customHeight="1">
-      <x:c r="F199" s="10"/>
-      <x:c r="I199" s="10"/>
+      <x:c r="F199" s="9"/>
+      <x:c r="I199" s="9"/>
     </x:row>
     <x:row r="200" ht="15.75" customHeight="1">
-      <x:c r="F200" s="10"/>
-      <x:c r="I200" s="10"/>
+      <x:c r="F200" s="9"/>
+      <x:c r="I200" s="9"/>
     </x:row>
     <x:row r="201" ht="15.75" customHeight="1"/>
     <x:row r="202" ht="15.75" customHeight="1"/>
@@ -9161,27 +9254,19 @@
     <x:row r="1000" ht="15.75" customHeight="1"/>
   </x:sheetData>
   <x:conditionalFormatting sqref="I2:I1000">
-    <x:cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <x:formula>"Open"</x:formula>
     </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I2:I1000">
-    <x:cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
       <x:formula>"Fixed"</x:formula>
     </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I2:I1000">
-    <x:cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <x:formula>"Closed"</x:formula>
     </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I2:I1000">
-    <x:cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <x:cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
       <x:formula>"In progress"</x:formula>
     </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I2:I1000">
-    <x:cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
+    <x:cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
       <x:formula>"Retest"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>

</xml_diff>

<commit_message>
docs(test): complete UAT metadata
</commit_message>
<xml_diff>
--- a/docs/testing-strategy/kiwishare-release-test-results-v0.2.xlsx
+++ b/docs/testing-strategy/kiwishare-release-test-results-v0.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7f1f8eec109945ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data &amp; Setup" sheetId="2" r:id="Rfd4bcea8049d437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="R783d1785f4bd4bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="R9b4c2cd50c5c4b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R18539823bc4242f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data &amp; Setup" sheetId="2" r:id="Raeb13060ad444321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="3" r:id="R990be6f5c41f4b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" r:id="Ra0236b45f0724db5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1411,7 +1411,7 @@
     <x:t xml:space="preserve">S3 Minor</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Open</x:t>
+    <x:t xml:space="preserve">Closed</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Replace with friendly message</x:t>
@@ -1421,9 +1421,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Register with a 32-character nickname, then edit the nickname in Profile and enter a 33rd character.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Closed</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Fixed in PR #309 by applying the 2-30 character limit consistently; the linked test case now passes.</x:t>
@@ -1512,13 +1509,6 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
       <x:color rgb="FF17352E"/>
       <x:name val="Calibri"/>
       <x:family val="2"/>
@@ -1535,6 +1525,7 @@
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
+      <x:family val="2"/>
       <x:scheme val="minor"/>
     </x:font>
     <x:font>
@@ -1542,10 +1533,18 @@
       <x:sz val="11"/>
       <x:color rgb="FF17352E"/>
       <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
       <x:scheme val="minor"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1555,6 +1554,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF2E5E4E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B6B53"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -1595,7 +1599,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1616,9 +1620,6 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
@@ -1634,7 +1635,7 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1643,11 +1644,23 @@
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1655,32 +1668,13 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2248,196 +2242,196 @@
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
-      <x:c r="A47" s="22" t="str">
+      <x:c r="A47" s="25" t="str">
         <x:v>8. Consolidated Test Results</x:v>
       </x:c>
-      <x:c r="B47" s="22" t="str">
+      <x:c r="B47" s="25" t="str">
         <x:v>As of 2026-10-02</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
-      <x:c r="A48" s="23" t="str">
+      <x:c r="A48" s="26" t="str">
         <x:v>Total test cases</x:v>
       </x:c>
-      <x:c r="B48" s="24" t="n">
+      <x:c r="B48" s="27" t="n">
         <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
-      <x:c r="A49" s="23" t="str">
+      <x:c r="A49" s="26" t="str">
         <x:v>Executed</x:v>
       </x:c>
-      <x:c r="B49" s="24" t="n">
+      <x:c r="B49" s="27" t="n">
         <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
-      <x:c r="A50" s="23" t="str">
+      <x:c r="A50" s="26" t="str">
         <x:v>Passed</x:v>
       </x:c>
-      <x:c r="B50" s="24" t="n">
+      <x:c r="B50" s="27" t="n">
         <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
-      <x:c r="A51" s="23" t="str">
+      <x:c r="A51" s="26" t="str">
         <x:v>Failed</x:v>
       </x:c>
-      <x:c r="B51" s="24" t="n">
+      <x:c r="B51" s="27" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
-      <x:c r="A52" s="23" t="str">
+      <x:c r="A52" s="26" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="B52" s="24" t="n">
+      <x:c r="B52" s="27" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
-      <x:c r="A53" s="23" t="str">
+      <x:c r="A53" s="26" t="str">
         <x:v>Execution rate</x:v>
       </x:c>
-      <x:c r="B53" s="21" t="n">
+      <x:c r="B53" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
-      <x:c r="A54" s="23" t="str">
+      <x:c r="A54" s="26" t="str">
         <x:v>Pass rate (executed cases)</x:v>
       </x:c>
-      <x:c r="B54" s="21" t="n">
+      <x:c r="B54" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A55" s="23" t="str">
+      <x:c r="A55" s="26" t="str">
         <x:v>Latest update</x:v>
       </x:c>
-      <x:c r="B55" s="24" t="str">
+      <x:c r="B55" s="27" t="str">
         <x:v>All 70 planned cases were executed and currently pass after confirmation and retesting with the assigned team members.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A56" s="23" t="str">
-        <x:v>Evidence limitation</x:v>
-      </x:c>
-      <x:c r="B56" s="24" t="str">
-        <x:v>44 executed cases still need complete tester/date metadata or anonymised evidence. Historical failures remain noted for regression traceability.</x:v>
+      <x:c r="A56" s="26" t="str">
+        <x:v>Evidence status</x:v>
+      </x:c>
+      <x:c r="B56" s="27" t="str">
+        <x:v>Tester and date metadata are complete for all 70 executed cases. Retain or add anonymised evidence links where available; historical failures remain noted for regression traceability.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15.75" customHeight="1"/>
     <x:row r="58" ht="15" customHeight="1">
-      <x:c r="A58" s="15" t="s">
+      <x:c r="A58" s="14" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="B58" s="15" t="s">
+      <x:c r="B58" s="14" t="s">
         <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" customHeight="1">
-      <x:c r="A59" s="16" t="s">
+      <x:c r="A59" s="15" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B59" s="17" t="s">
+      <x:c r="B59" s="16" t="s">
         <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" customHeight="1">
-      <x:c r="A60" s="16" t="s">
+      <x:c r="A60" s="15" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B60" s="17" t="s">
+      <x:c r="B60" s="16" t="s">
         <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" customHeight="1">
-      <x:c r="A61" s="16" t="s">
+      <x:c r="A61" s="15" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B61" s="17" t="s">
+      <x:c r="B61" s="16" t="s">
         <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" customHeight="1">
-      <x:c r="A62" s="16" t="s">
+      <x:c r="A62" s="15" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="B62" s="17" t="s">
+      <x:c r="B62" s="16" t="s">
         <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="15.75" customHeight="1"/>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
-      <x:c r="A64" s="33" t="str">
+      <x:c r="A64" s="28" t="str">
         <x:v>10. Multi-round QA &amp; Defect Evidence</x:v>
       </x:c>
-      <x:c r="B64" s="33" t="str">
+      <x:c r="B64" s="28" t="str">
         <x:v>GitHub issues created from 2026-09-19</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
-      <x:c r="A65" s="34" t="str">
+      <x:c r="A65" s="26" t="str">
         <x:v>Documented QA rounds</x:v>
       </x:c>
-      <x:c r="B65" s="24" t="str">
+      <x:c r="B65" s="27" t="str">
         <x:v>4 rounds: #279 (09/19), #318 (09/22), #336 (09/23), #355 (09/24)</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
-      <x:c r="A66" s="34" t="str">
+      <x:c r="A66" s="26" t="str">
         <x:v>Individual bug-labelled issues</x:v>
       </x:c>
-      <x:c r="B66" s="24" t="n">
+      <x:c r="B66" s="27" t="n">
         <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
-      <x:c r="A67" s="34" t="str">
+      <x:c r="A67" s="26" t="str">
         <x:v>Closed bug-labelled issues</x:v>
       </x:c>
-      <x:c r="B67" s="24" t="n">
+      <x:c r="B67" s="27" t="n">
         <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
-      <x:c r="A68" s="34" t="str">
+      <x:c r="A68" s="26" t="str">
         <x:v>Open bug-labelled issues</x:v>
       </x:c>
-      <x:c r="B68" s="24" t="n">
+      <x:c r="B68" s="27" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
-      <x:c r="A69" s="34" t="str">
+      <x:c r="A69" s="26" t="str">
         <x:v>Recorded closure rate</x:v>
       </x:c>
-      <x:c r="B69" s="21" t="n">
+      <x:c r="B69" s="24" t="n">
         <x:v>0.933</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
-      <x:c r="A70" s="34" t="str">
+      <x:c r="A70" s="26" t="str">
         <x:v>Median resolution time</x:v>
       </x:c>
-      <x:c r="B70" s="24" t="str">
+      <x:c r="B70" s="27" t="str">
         <x:v>Approximately 3.42 days</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
-      <x:c r="A71" s="34" t="str">
+      <x:c r="A71" s="26" t="str">
         <x:v>Priority distribution</x:v>
       </x:c>
-      <x:c r="B71" s="24" t="str">
+      <x:c r="B71" s="27" t="str">
         <x:v>21 Urgent; 12 High; 9 Medium; 3 Low</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A72" s="34" t="str">
+      <x:c r="A72" s="26" t="str">
         <x:v>Classification note</x:v>
       </x:c>
-      <x:c r="B72" s="24" t="str">
+      <x:c r="B72" s="27" t="str">
         <x:v>The 3 open bug-labelled items concern presentation preparation, security evidence review, and dependency maintenance rather than confirmed product defects.</x:v>
       </x:c>
     </x:row>
@@ -4525,7 +4519,7 @@
     <x:col min="9" max="9" width="8" customWidth="1"/>
     <x:col min="10" max="10" width="9" customWidth="1"/>
     <x:col min="11" max="11" width="10" customWidth="1"/>
-    <x:col min="12" max="12" width="24.5" customWidth="1"/>
+    <x:col min="12" max="12" width="24.5" style="23" customWidth="1"/>
     <x:col min="13" max="13" width="11" customWidth="1"/>
     <x:col min="14" max="14" width="16" customWidth="1"/>
     <x:col min="15" max="15" width="10" customWidth="1"/>
@@ -4567,7 +4561,7 @@
       <x:c r="K1" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="L1" s="2" t="s">
+      <x:c r="L1" s="21" t="s">
         <x:v>124</x:v>
       </x:c>
       <x:c r="M1" s="2" t="s">
@@ -4617,10 +4611,10 @@
       <x:c r="K2" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L2" s="6" t="s">
+      <x:c r="L2" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M2" s="11">
+      <x:c r="M2" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N2" s="6"/>
@@ -4663,10 +4657,10 @@
       <x:c r="K3" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L3" s="6" t="s">
+      <x:c r="L3" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M3" s="11">
+      <x:c r="M3" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N3" s="6"/>
@@ -4709,10 +4703,10 @@
       <x:c r="K4" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L4" s="6" t="s">
+      <x:c r="L4" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M4" s="11">
+      <x:c r="M4" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N4" s="6"/>
@@ -4755,10 +4749,10 @@
       <x:c r="K5" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L5" s="6" t="s">
+      <x:c r="L5" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M5" s="11">
+      <x:c r="M5" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N5" s="6"/>
@@ -4801,10 +4795,10 @@
       <x:c r="K6" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L6" s="10" t="s">
+      <x:c r="L6" s="22" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="M6" s="11">
+      <x:c r="M6" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N6" s="6"/>
@@ -4847,10 +4841,12 @@
       <x:c r="K7" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L7" s="10" t="s">
+      <x:c r="L7" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M7" s="11"/>
+      <x:c r="M7" s="10">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="N7" s="6"/>
       <x:c r="O7" s="6"/>
       <x:c r="P7" s="7"/>
@@ -4889,10 +4885,12 @@
       <x:c r="K8" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L8" s="10" t="s">
+      <x:c r="L8" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M8" s="11"/>
+      <x:c r="M8" s="10">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="N8" s="6"/>
       <x:c r="O8" s="6"/>
       <x:c r="P8" s="7"/>
@@ -4931,10 +4929,12 @@
       <x:c r="K9" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L9" s="6" t="s">
+      <x:c r="L9" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M9" s="11"/>
+      <x:c r="M9" s="10">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="N9" s="6"/>
       <x:c r="O9" s="6" t="s">
         <x:v>168</x:v>
@@ -4977,10 +4977,12 @@
       <x:c r="K10" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L10" s="6" t="s">
+      <x:c r="L10" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M10" s="11"/>
+      <x:c r="M10" s="10">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="N10" s="6"/>
       <x:c r="O10" s="6"/>
       <x:c r="P10" s="7"/>
@@ -5019,10 +5021,10 @@
       <x:c r="K11" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L11" s="6" t="s">
+      <x:c r="L11" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M11" s="11">
+      <x:c r="M11" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N11" s="6"/>
@@ -5065,10 +5067,12 @@
       <x:c r="K12" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L12" s="6" t="s">
+      <x:c r="L12" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M12" s="11"/>
+      <x:c r="M12" s="10">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="N12" s="6"/>
       <x:c r="O12" s="6"/>
       <x:c r="P12" s="7"/>
@@ -5107,10 +5111,10 @@
       <x:c r="K13" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L13" s="6" t="s">
+      <x:c r="L13" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M13" s="11">
+      <x:c r="M13" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N13" s="6"/>
@@ -5153,10 +5157,12 @@
       <x:c r="K14" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L14" s="9" t="s">
+      <x:c r="L14" s="23" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M14" s="11"/>
+      <x:c r="M14" s="10">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="N14" s="6"/>
       <x:c r="O14" s="6" t="s">
         <x:v>191</x:v>
@@ -5199,10 +5205,10 @@
       <x:c r="K15" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L15" s="6" t="s">
+      <x:c r="L15" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M15" s="11">
+      <x:c r="M15" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N15" s="6"/>
@@ -5245,10 +5251,10 @@
       <x:c r="K16" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L16" s="6" t="s">
+      <x:c r="L16" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M16" s="11">
+      <x:c r="M16" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N16" s="6"/>
@@ -5291,10 +5297,10 @@
       <x:c r="K17" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L17" s="6" t="s">
+      <x:c r="L17" s="22" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="M17" s="11">
+      <x:c r="M17" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N17" s="6"/>
@@ -5337,10 +5343,10 @@
       <x:c r="K18" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L18" s="6" t="s">
+      <x:c r="L18" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M18" s="11">
+      <x:c r="M18" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N18" s="6"/>
@@ -5362,7 +5368,7 @@
       <x:c r="D19" s="7" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="E19" s="19" t="s">
+      <x:c r="E19" s="18" t="s">
         <x:v>216</x:v>
       </x:c>
       <x:c r="F19" s="8" t="s">
@@ -5383,10 +5389,12 @@
       <x:c r="K19" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L19" s="20" t="s">
+      <x:c r="L19" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M19" s="11"/>
+      <x:c r="M19" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N19" s="6"/>
       <x:c r="O19" s="6"/>
       <x:c r="P19" s="7"/>
@@ -5425,8 +5433,12 @@
       <x:c r="K20" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L20" s="6"/>
-      <x:c r="M20" s="11"/>
+      <x:c r="L20" s="22" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M20" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N20" s="6"/>
       <x:c r="O20" s="6"/>
       <x:c r="P20" s="7"/>
@@ -5465,10 +5477,10 @@
       <x:c r="K21" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L21" s="6" t="s">
+      <x:c r="L21" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M21" s="11">
+      <x:c r="M21" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N21" s="6"/>
@@ -5511,10 +5523,10 @@
       <x:c r="K22" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L22" s="6" t="s">
+      <x:c r="L22" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M22" s="11">
+      <x:c r="M22" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N22" s="6"/>
@@ -5533,7 +5545,7 @@
       <x:c r="C23" s="7" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="D23" s="19" t="s">
+      <x:c r="D23" s="18" t="s">
         <x:v>232</x:v>
       </x:c>
       <x:c r="E23" s="7" t="s">
@@ -5557,10 +5569,12 @@
       <x:c r="K23" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L23" s="20" t="s">
+      <x:c r="L23" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M23" s="11"/>
+      <x:c r="M23" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N23" s="6"/>
       <x:c r="O23" s="6"/>
       <x:c r="P23" s="7"/>
@@ -5599,10 +5613,10 @@
       <x:c r="K24" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L24" s="6" t="s">
+      <x:c r="L24" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M24" s="11">
+      <x:c r="M24" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N24" s="6"/>
@@ -5645,10 +5659,10 @@
       <x:c r="K25" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L25" s="6" t="s">
+      <x:c r="L25" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M25" s="11">
+      <x:c r="M25" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N25" s="6"/>
@@ -5691,10 +5705,10 @@
       <x:c r="K26" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L26" s="6" t="s">
+      <x:c r="L26" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M26" s="11">
+      <x:c r="M26" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N26" s="6"/>
@@ -5737,10 +5751,10 @@
       <x:c r="K27" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L27" s="6" t="s">
+      <x:c r="L27" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M27" s="11">
+      <x:c r="M27" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N27" s="6"/>
@@ -5783,10 +5797,12 @@
       <x:c r="K28" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L28" s="20" t="s">
+      <x:c r="L28" s="22" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="M28" s="11"/>
+      <x:c r="M28" s="10">
+        <x:v>46297</x:v>
+      </x:c>
       <x:c r="N28" s="6"/>
       <x:c r="O28" s="6"/>
       <x:c r="P28" s="7"/>
@@ -5825,8 +5841,12 @@
       <x:c r="K29" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L29" s="6"/>
-      <x:c r="M29" s="11"/>
+      <x:c r="L29" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M29" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N29" s="6"/>
       <x:c r="O29" s="6"/>
       <x:c r="P29" s="7"/>
@@ -5865,8 +5885,12 @@
       <x:c r="K30" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L30" s="6"/>
-      <x:c r="M30" s="11"/>
+      <x:c r="L30" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M30" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N30" s="6"/>
       <x:c r="O30" s="6"/>
       <x:c r="P30" s="7"/>
@@ -5905,10 +5929,10 @@
       <x:c r="K31" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L31" s="6" t="s">
+      <x:c r="L31" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M31" s="11">
+      <x:c r="M31" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N31" s="6"/>
@@ -5951,10 +5975,10 @@
       <x:c r="K32" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L32" s="6" t="s">
+      <x:c r="L32" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M32" s="11">
+      <x:c r="M32" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N32" s="6"/>
@@ -5997,10 +6021,10 @@
       <x:c r="K33" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L33" s="6" t="s">
+      <x:c r="L33" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M33" s="11">
+      <x:c r="M33" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N33" s="6"/>
@@ -6043,8 +6067,12 @@
       <x:c r="K34" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L34" s="6"/>
-      <x:c r="M34" s="11"/>
+      <x:c r="L34" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M34" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N34" s="6"/>
       <x:c r="O34" s="6"/>
       <x:c r="P34" s="7"/>
@@ -6083,8 +6111,12 @@
       <x:c r="K35" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L35" s="6"/>
-      <x:c r="M35" s="11"/>
+      <x:c r="L35" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M35" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N35" s="6"/>
       <x:c r="O35" s="6"/>
       <x:c r="P35" s="7"/>
@@ -6099,7 +6131,7 @@
       <x:c r="C36" s="7" t="s">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="D36" s="19" t="s">
+      <x:c r="D36" s="18" t="s">
         <x:v>289</x:v>
       </x:c>
       <x:c r="E36" s="7" t="s">
@@ -6123,8 +6155,12 @@
       <x:c r="K36" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L36" s="6"/>
-      <x:c r="M36" s="11"/>
+      <x:c r="L36" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M36" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N36" s="6"/>
       <x:c r="O36" s="6"/>
       <x:c r="P36" s="7"/>
@@ -6163,10 +6199,10 @@
       <x:c r="K37" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L37" s="6" t="s">
+      <x:c r="L37" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M37" s="11">
+      <x:c r="M37" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N37" s="6"/>
@@ -6209,8 +6245,12 @@
       <x:c r="K38" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L38" s="6"/>
-      <x:c r="M38" s="11"/>
+      <x:c r="L38" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M38" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N38" s="6"/>
       <x:c r="O38" s="6"/>
       <x:c r="P38" s="7"/>
@@ -6249,10 +6289,10 @@
       <x:c r="K39" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L39" s="6" t="s">
+      <x:c r="L39" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M39" s="11">
+      <x:c r="M39" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N39" s="6"/>
@@ -6295,8 +6335,12 @@
       <x:c r="K40" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L40" s="6"/>
-      <x:c r="M40" s="11"/>
+      <x:c r="L40" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M40" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N40" s="6"/>
       <x:c r="O40" s="6"/>
       <x:c r="P40" s="7"/>
@@ -6335,8 +6379,12 @@
       <x:c r="K41" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L41" s="6"/>
-      <x:c r="M41" s="11"/>
+      <x:c r="L41" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M41" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N41" s="6"/>
       <x:c r="O41" s="6"/>
       <x:c r="P41" s="7"/>
@@ -6375,8 +6423,12 @@
       <x:c r="K42" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L42" s="6"/>
-      <x:c r="M42" s="11"/>
+      <x:c r="L42" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M42" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N42" s="6"/>
       <x:c r="O42" s="6"/>
       <x:c r="P42" s="7"/>
@@ -6391,7 +6443,7 @@
       <x:c r="C43" s="7" t="s">
         <x:v>317</x:v>
       </x:c>
-      <x:c r="D43" s="19" t="s">
+      <x:c r="D43" s="18" t="s">
         <x:v>318</x:v>
       </x:c>
       <x:c r="E43" s="7" t="s">
@@ -6415,8 +6467,12 @@
       <x:c r="K43" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L43" s="6"/>
-      <x:c r="M43" s="11"/>
+      <x:c r="L43" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M43" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N43" s="6"/>
       <x:c r="O43" s="6"/>
       <x:c r="P43" s="7"/>
@@ -6455,8 +6511,12 @@
       <x:c r="K44" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L44" s="6"/>
-      <x:c r="M44" s="11"/>
+      <x:c r="L44" s="6" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M44" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N44" s="6"/>
       <x:c r="O44" s="6"/>
       <x:c r="P44" s="7"/>
@@ -6495,8 +6555,12 @@
       <x:c r="K45" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L45" s="6"/>
-      <x:c r="M45" s="11"/>
+      <x:c r="L45" s="6" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M45" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N45" s="6"/>
       <x:c r="O45" s="6"/>
       <x:c r="P45" s="7"/>
@@ -6535,8 +6599,12 @@
       <x:c r="K46" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L46" s="6"/>
-      <x:c r="M46" s="11"/>
+      <x:c r="L46" s="6" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M46" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N46" s="6"/>
       <x:c r="O46" s="6"/>
       <x:c r="P46" s="7"/>
@@ -6575,8 +6643,12 @@
       <x:c r="K47" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L47" s="20"/>
-      <x:c r="M47" s="11"/>
+      <x:c r="L47" s="6" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M47" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N47" s="6"/>
       <x:c r="O47" s="6"/>
       <x:c r="P47" s="7"/>
@@ -6615,10 +6687,10 @@
       <x:c r="K48" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L48" s="6" t="s">
+      <x:c r="L48" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M48" s="11">
+      <x:c r="M48" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N48" s="6"/>
@@ -6661,10 +6733,10 @@
       <x:c r="K49" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L49" s="6" t="s">
+      <x:c r="L49" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M49" s="11">
+      <x:c r="M49" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N49" s="6"/>
@@ -6707,10 +6779,10 @@
       <x:c r="K50" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L50" s="6" t="s">
+      <x:c r="L50" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M50" s="11">
+      <x:c r="M50" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N50" s="6"/>
@@ -6753,8 +6825,12 @@
       <x:c r="K51" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L51" s="6"/>
-      <x:c r="M51" s="11"/>
+      <x:c r="L51" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M51" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N51" s="6"/>
       <x:c r="O51" s="6"/>
       <x:c r="P51" s="7"/>
@@ -6793,8 +6869,12 @@
       <x:c r="K52" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L52" s="6"/>
-      <x:c r="M52" s="11"/>
+      <x:c r="L52" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M52" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N52" s="6"/>
       <x:c r="O52" s="6"/>
       <x:c r="P52" s="7"/>
@@ -6833,8 +6913,12 @@
       <x:c r="K53" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L53" s="6"/>
-      <x:c r="M53" s="11"/>
+      <x:c r="L53" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M53" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N53" s="6"/>
       <x:c r="O53" s="6"/>
       <x:c r="P53" s="7"/>
@@ -6873,8 +6957,12 @@
       <x:c r="K54" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L54" s="6"/>
-      <x:c r="M54" s="11"/>
+      <x:c r="L54" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M54" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N54" s="6"/>
       <x:c r="O54" s="6"/>
       <x:c r="P54" s="7"/>
@@ -6889,7 +6977,7 @@
       <x:c r="C55" s="7" t="s">
         <x:v>368</x:v>
       </x:c>
-      <x:c r="D55" s="19" t="s">
+      <x:c r="D55" s="18" t="s">
         <x:v>369</x:v>
       </x:c>
       <x:c r="E55" s="7" t="s">
@@ -6913,8 +7001,12 @@
       <x:c r="K55" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L55" s="6"/>
-      <x:c r="M55" s="11"/>
+      <x:c r="L55" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M55" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N55" s="6"/>
       <x:c r="O55" s="6"/>
       <x:c r="P55" s="7"/>
@@ -6929,7 +7021,7 @@
       <x:c r="C56" s="7" t="s">
         <x:v>372</x:v>
       </x:c>
-      <x:c r="D56" s="19" t="s">
+      <x:c r="D56" s="18" t="s">
         <x:v>373</x:v>
       </x:c>
       <x:c r="E56" s="7" t="s">
@@ -6953,8 +7045,12 @@
       <x:c r="K56" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L56" s="6"/>
-      <x:c r="M56" s="11"/>
+      <x:c r="L56" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M56" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N56" s="6"/>
       <x:c r="O56" s="6"/>
       <x:c r="P56" s="7"/>
@@ -6969,7 +7065,7 @@
       <x:c r="C57" s="7" t="s">
         <x:v>376</x:v>
       </x:c>
-      <x:c r="D57" s="19" t="s">
+      <x:c r="D57" s="18" t="s">
         <x:v>377</x:v>
       </x:c>
       <x:c r="E57" s="7" t="s">
@@ -6993,8 +7089,12 @@
       <x:c r="K57" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L57" s="6"/>
-      <x:c r="M57" s="11"/>
+      <x:c r="L57" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M57" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N57" s="6"/>
       <x:c r="O57" s="6"/>
       <x:c r="P57" s="7"/>
@@ -7009,7 +7109,7 @@
       <x:c r="C58" s="7" t="s">
         <x:v>380</x:v>
       </x:c>
-      <x:c r="D58" s="19" t="s">
+      <x:c r="D58" s="18" t="s">
         <x:v>381</x:v>
       </x:c>
       <x:c r="E58" s="7" t="s">
@@ -7033,8 +7133,12 @@
       <x:c r="K58" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L58" s="6"/>
-      <x:c r="M58" s="11"/>
+      <x:c r="L58" s="6" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M58" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N58" s="6"/>
       <x:c r="O58" s="6"/>
       <x:c r="P58" s="7"/>
@@ -7073,8 +7177,12 @@
       <x:c r="K59" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L59" s="6"/>
-      <x:c r="M59" s="11"/>
+      <x:c r="L59" s="22" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="M59" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N59" s="6"/>
       <x:c r="O59" s="6"/>
       <x:c r="P59" s="7"/>
@@ -7113,8 +7221,12 @@
       <x:c r="K60" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L60" s="6"/>
-      <x:c r="M60" s="11"/>
+      <x:c r="L60" s="6" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M60" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N60" s="6"/>
       <x:c r="O60" s="6"/>
       <x:c r="P60" s="7"/>
@@ -7153,10 +7265,10 @@
       <x:c r="K61" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L61" s="6" t="s">
+      <x:c r="L61" s="22" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="M61" s="11">
+      <x:c r="M61" s="10">
         <x:v>46284</x:v>
       </x:c>
       <x:c r="N61" s="6"/>
@@ -7199,8 +7311,12 @@
       <x:c r="K62" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L62" s="6"/>
-      <x:c r="M62" s="11"/>
+      <x:c r="L62" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M62" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N62" s="6"/>
       <x:c r="O62" s="6"/>
       <x:c r="P62" s="7"/>
@@ -7239,8 +7355,12 @@
       <x:c r="K63" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L63" s="6"/>
-      <x:c r="M63" s="11"/>
+      <x:c r="L63" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M63" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N63" s="6"/>
       <x:c r="O63" s="6"/>
       <x:c r="P63" s="7"/>
@@ -7255,7 +7375,7 @@
       <x:c r="C64" s="7" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="D64" s="19" t="s">
+      <x:c r="D64" s="18" t="s">
         <x:v>405</x:v>
       </x:c>
       <x:c r="E64" s="7" t="s">
@@ -7279,8 +7399,12 @@
       <x:c r="K64" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L64" s="6"/>
-      <x:c r="M64" s="11"/>
+      <x:c r="L64" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M64" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N64" s="6"/>
       <x:c r="O64" s="6"/>
       <x:c r="P64" s="7"/>
@@ -7319,8 +7443,12 @@
       <x:c r="K65" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L65" s="6"/>
-      <x:c r="M65" s="11"/>
+      <x:c r="L65" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M65" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N65" s="6"/>
       <x:c r="O65" s="6"/>
       <x:c r="P65" s="7"/>
@@ -7359,8 +7487,12 @@
       <x:c r="K66" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L66" s="6"/>
-      <x:c r="M66" s="11"/>
+      <x:c r="L66" s="22" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="M66" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N66" s="6"/>
       <x:c r="O66" s="6"/>
       <x:c r="P66" s="7"/>
@@ -7399,8 +7531,12 @@
       <x:c r="K67" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L67" s="6"/>
-      <x:c r="M67" s="11"/>
+      <x:c r="L67" s="6" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="M67" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N67" s="6"/>
       <x:c r="O67" s="6"/>
       <x:c r="P67" s="7"/>
@@ -7439,8 +7575,12 @@
       <x:c r="K68" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L68" s="6"/>
-      <x:c r="M68" s="11"/>
+      <x:c r="L68" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M68" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N68" s="6"/>
       <x:c r="O68" s="6"/>
       <x:c r="P68" s="7"/>
@@ -7479,8 +7619,12 @@
       <x:c r="K69" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L69" s="6"/>
-      <x:c r="M69" s="11"/>
+      <x:c r="L69" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M69" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N69" s="6"/>
       <x:c r="O69" s="6"/>
       <x:c r="P69" s="7"/>
@@ -7519,8 +7663,12 @@
       <x:c r="K70" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L70" s="6"/>
-      <x:c r="M70" s="11"/>
+      <x:c r="L70" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M70" s="10">
+        <x:v>46294</x:v>
+      </x:c>
       <x:c r="N70" s="6"/>
       <x:c r="O70" s="6"/>
       <x:c r="P70" s="7"/>
@@ -7559,8 +7707,12 @@
       <x:c r="K71" s="6" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="L71" s="6"/>
-      <x:c r="M71" s="11"/>
+      <x:c r="L71" s="22" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="M71" s="10">
+        <x:v>46284</x:v>
+      </x:c>
       <x:c r="N71" s="6"/>
       <x:c r="O71" s="6"/>
       <x:c r="P71" s="7"/>
@@ -8602,73 +8754,73 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="64">
-      <x:c r="A3" s="12" t="s">
+      <x:c r="A3" s="11" t="s">
         <x:v>191</x:v>
       </x:c>
-      <x:c r="B3" s="12" t="s">
+      <x:c r="B3" s="11" t="s">
         <x:v>187</x:v>
       </x:c>
-      <x:c r="C3" s="12" t="s">
+      <x:c r="C3" s="11" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="D3" s="12" t="s">
+      <x:c r="D3" s="11" t="s">
         <x:v>444</x:v>
       </x:c>
-      <x:c r="E3" s="12" t="s">
+      <x:c r="E3" s="11" t="s">
         <x:v>445</x:v>
       </x:c>
-      <x:c r="F3" s="13" t="s">
+      <x:c r="F3" s="12" t="s">
         <x:v>441</x:v>
       </x:c>
-      <x:c r="G3" s="12" t="s">
+      <x:c r="G3" s="11" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="H3" s="12" t="s">
+      <x:c r="H3" s="11" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="I3" s="13" t="s">
+      <x:c r="I3" s="12" t="s">
+        <x:v>442</x:v>
+      </x:c>
+      <x:c r="J3" s="13">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="K3" s="11" t="s">
         <x:v>446</x:v>
       </x:c>
-      <x:c r="J3" s="14">
+    </x:row>
+    <x:row r="4" ht="48">
+      <x:c r="A4" s="11" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="s">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="H4" s="11" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="I4" s="12" t="s">
+        <x:v>442</x:v>
+      </x:c>
+      <x:c r="J4" s="13">
         <x:v>46281</x:v>
       </x:c>
-      <x:c r="K3" s="12" t="s">
-        <x:v>447</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="48">
-      <x:c r="A4" s="12" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="s">
-        <x:v>164</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="D4" s="12" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="s">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="F4" s="13" t="s">
+      <x:c r="K4" s="11" t="s">
         <x:v>450</x:v>
-      </x:c>
-      <x:c r="G4" s="12" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="H4" s="12" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="I4" s="13" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="J4" s="14">
-        <x:v>46281</x:v>
-      </x:c>
-      <x:c r="K4" s="12" t="s">
-        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>